<commit_message>
Discovery: full-UAE run plan + 900/hour pacing; tracker auto status
- serp-discovery.ts: named runs (pilot-dubai, full-uae: 60 categories x
  51 areas / 3 cities), 4 workers, retries, paced to 900 searches/hour
  (plan limit is 1,000/hour, which the first full-run attempt hit).
- data_tracker.py: Status refreshes automatically (Not started /
  Discovering / Manual list for non-map categories) unless set by hand.
- Tracker refreshed: 1,014 searches, 13,842 places in 13 categories.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reviewencer-data-tracker.xlsx
+++ b/docs/Reviewencer-data-tracker.xlsx
@@ -331,7 +331,7 @@
     </comment>
     <comment ref="B18" authorId="0" shapeId="0">
       <text>
-        <t>Read from the SerpAPI account page at 2026-10-21 11:41 (free lookup). Refreshes when the tracker is regenerated.</t>
+        <t>Read from the SerpAPI account page at 2026-10-21 11:52 (free lookup). Refreshes when the tracker is regenerated.</t>
       </text>
     </comment>
   </commentList>
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-21 11:41 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
+          <t>Generated 2026-10-21 11:52 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
         </is>
       </c>
     </row>
@@ -877,25 +877,25 @@
         <v>0</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>50</v>
+        <v>152</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>965</v>
+        <v>2121</v>
       </c>
       <c r="Q6" s="12" t="n">
-        <v>736</v>
+        <v>1552</v>
       </c>
       <c r="R6" s="12" t="n">
-        <v>942</v>
+        <v>2078</v>
       </c>
       <c r="S6" s="12" t="n">
-        <v>957</v>
+        <v>2091</v>
       </c>
       <c r="T6" s="12" t="n">
-        <v>965</v>
+        <v>2121</v>
       </c>
       <c r="U6" s="12" t="n">
-        <v>957</v>
+        <v>2065</v>
       </c>
       <c r="V6" s="13">
         <f>IFERROR(SUM(Q6:U6)/(5*P6),0)</f>
@@ -903,7 +903,7 @@
       </c>
       <c r="W6" s="14" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X6" s="15" t="n"/>
@@ -964,25 +964,25 @@
         <v>0</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>0</v>
+        <v>1740</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>0</v>
+        <v>1241</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>0</v>
+        <v>1654</v>
       </c>
       <c r="S7" s="12" t="n">
-        <v>0</v>
+        <v>1695</v>
       </c>
       <c r="T7" s="12" t="n">
-        <v>0</v>
+        <v>1740</v>
       </c>
       <c r="U7" s="12" t="n">
-        <v>0</v>
+        <v>1592</v>
       </c>
       <c r="V7" s="13">
         <f>IFERROR(SUM(Q7:U7)/(5*P7),0)</f>
@@ -990,7 +990,7 @@
       </c>
       <c r="W7" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X7" s="15" t="n"/>
@@ -1051,25 +1051,25 @@
         <v>0</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="Q8" s="12" t="n">
-        <v>0</v>
+        <v>679</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>0</v>
+        <v>880</v>
       </c>
       <c r="S8" s="12" t="n">
-        <v>0</v>
+        <v>892</v>
       </c>
       <c r="T8" s="12" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="U8" s="12" t="n">
-        <v>0</v>
+        <v>877</v>
       </c>
       <c r="V8" s="13">
         <f>IFERROR(SUM(Q8:U8)/(5*P8),0)</f>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="W8" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X8" s="15" t="n"/>
@@ -1138,25 +1138,25 @@
         <v>0</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>0</v>
+        <v>729</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>0</v>
+        <v>534</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>0</v>
+        <v>702</v>
       </c>
       <c r="S9" s="12" t="n">
-        <v>0</v>
+        <v>717</v>
       </c>
       <c r="T9" s="12" t="n">
-        <v>0</v>
+        <v>729</v>
       </c>
       <c r="U9" s="12" t="n">
-        <v>0</v>
+        <v>646</v>
       </c>
       <c r="V9" s="13">
         <f>IFERROR(SUM(Q9:U9)/(5*P9),0)</f>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="W9" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X9" s="15" t="n"/>
@@ -1225,25 +1225,25 @@
         <v>0</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P10" s="12" t="n">
-        <v>0</v>
+        <v>809</v>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>0</v>
+        <v>616</v>
       </c>
       <c r="R10" s="12" t="n">
-        <v>0</v>
+        <v>776</v>
       </c>
       <c r="S10" s="12" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="T10" s="12" t="n">
-        <v>0</v>
+        <v>809</v>
       </c>
       <c r="U10" s="12" t="n">
-        <v>0</v>
+        <v>742</v>
       </c>
       <c r="V10" s="13">
         <f>IFERROR(SUM(Q10:U10)/(5*P10),0)</f>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="W10" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X10" s="15" t="n"/>
@@ -1573,25 +1573,25 @@
         <v>0</v>
       </c>
       <c r="O14" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P14" s="12" t="n">
-        <v>0</v>
+        <v>817</v>
       </c>
       <c r="Q14" s="12" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="R14" s="12" t="n">
-        <v>0</v>
+        <v>776</v>
       </c>
       <c r="S14" s="12" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="T14" s="12" t="n">
-        <v>0</v>
+        <v>817</v>
       </c>
       <c r="U14" s="12" t="n">
-        <v>0</v>
+        <v>709</v>
       </c>
       <c r="V14" s="13">
         <f>IFERROR(SUM(Q14:U14)/(5*P14),0)</f>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="W14" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X14" s="15" t="n"/>
@@ -1660,25 +1660,25 @@
         <v>0</v>
       </c>
       <c r="O15" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P15" s="12" t="n">
-        <v>0</v>
+        <v>517</v>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>0</v>
+        <v>301</v>
       </c>
       <c r="R15" s="12" t="n">
-        <v>0</v>
+        <v>470</v>
       </c>
       <c r="S15" s="12" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="T15" s="12" t="n">
-        <v>0</v>
+        <v>517</v>
       </c>
       <c r="U15" s="12" t="n">
-        <v>0</v>
+        <v>404</v>
       </c>
       <c r="V15" s="13">
         <f>IFERROR(SUM(Q15:U15)/(5*P15),0)</f>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="W15" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X15" s="15" t="n"/>
@@ -1834,25 +1834,25 @@
         <v>0</v>
       </c>
       <c r="O17" s="12" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="P17" s="12" t="n">
-        <v>0</v>
+        <v>1375</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>0</v>
+        <v>1137</v>
       </c>
       <c r="R17" s="12" t="n">
-        <v>0</v>
+        <v>1325</v>
       </c>
       <c r="S17" s="12" t="n">
-        <v>0</v>
+        <v>1308</v>
       </c>
       <c r="T17" s="12" t="n">
-        <v>0</v>
+        <v>1375</v>
       </c>
       <c r="U17" s="12" t="n">
-        <v>0</v>
+        <v>1123</v>
       </c>
       <c r="V17" s="13">
         <f>IFERROR(SUM(Q17:U17)/(5*P17),0)</f>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="W17" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X17" s="15" t="n"/>
@@ -2182,25 +2182,25 @@
         <v>0</v>
       </c>
       <c r="O21" s="12" t="n">
-        <v>47</v>
+        <v>139</v>
       </c>
       <c r="P21" s="12" t="n">
-        <v>656</v>
+        <v>1144</v>
       </c>
       <c r="Q21" s="12" t="n">
-        <v>578</v>
+        <v>965</v>
       </c>
       <c r="R21" s="12" t="n">
-        <v>647</v>
+        <v>1130</v>
       </c>
       <c r="S21" s="12" t="n">
-        <v>644</v>
+        <v>1124</v>
       </c>
       <c r="T21" s="12" t="n">
-        <v>656</v>
+        <v>1144</v>
       </c>
       <c r="U21" s="12" t="n">
-        <v>548</v>
+        <v>969</v>
       </c>
       <c r="V21" s="13">
         <f>IFERROR(SUM(Q21:U21)/(5*P21),0)</f>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="W21" s="14" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X21" s="15" t="n"/>
@@ -2269,25 +2269,25 @@
         <v>0</v>
       </c>
       <c r="O22" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P22" s="12" t="n">
-        <v>0</v>
+        <v>760</v>
       </c>
       <c r="Q22" s="12" t="n">
-        <v>0</v>
+        <v>643</v>
       </c>
       <c r="R22" s="12" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="S22" s="12" t="n">
-        <v>0</v>
+        <v>749</v>
       </c>
       <c r="T22" s="12" t="n">
-        <v>0</v>
+        <v>760</v>
       </c>
       <c r="U22" s="12" t="n">
-        <v>0</v>
+        <v>615</v>
       </c>
       <c r="V22" s="13">
         <f>IFERROR(SUM(Q22:U22)/(5*P22),0)</f>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="W22" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X22" s="15" t="n"/>
@@ -2356,25 +2356,25 @@
         <v>0</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P23" s="12" t="n">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="R23" s="12" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="S23" s="12" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="T23" s="12" t="n">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="U23" s="12" t="n">
-        <v>0</v>
+        <v>183</v>
       </c>
       <c r="V23" s="13">
         <f>IFERROR(SUM(Q23:U23)/(5*P23),0)</f>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="W23" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X23" s="15" t="n"/>
@@ -2443,25 +2443,25 @@
         <v>0</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="P24" s="12" t="n">
-        <v>0</v>
+        <v>1506</v>
       </c>
       <c r="Q24" s="12" t="n">
-        <v>0</v>
+        <v>1099</v>
       </c>
       <c r="R24" s="12" t="n">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="S24" s="12" t="n">
-        <v>0</v>
+        <v>1483</v>
       </c>
       <c r="T24" s="12" t="n">
-        <v>0</v>
+        <v>1506</v>
       </c>
       <c r="U24" s="12" t="n">
-        <v>0</v>
+        <v>1308</v>
       </c>
       <c r="V24" s="13">
         <f>IFERROR(SUM(Q24:U24)/(5*P24),0)</f>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="W24" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X24" s="15" t="n"/>
@@ -3574,25 +3574,25 @@
         <v>0</v>
       </c>
       <c r="O37" s="12" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="P37" s="12" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="Q37" s="12" t="n">
-        <v>0</v>
+        <v>781</v>
       </c>
       <c r="R37" s="12" t="n">
-        <v>0</v>
+        <v>1096</v>
       </c>
       <c r="S37" s="12" t="n">
-        <v>0</v>
+        <v>1110</v>
       </c>
       <c r="T37" s="12" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="U37" s="12" t="n">
-        <v>0</v>
+        <v>912</v>
       </c>
       <c r="V37" s="13">
         <f>IFERROR(SUM(Q37:U37)/(5*P37),0)</f>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="W37" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X37" s="15" t="n"/>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="W43" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X43" s="15" t="n"/>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="W49" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X49" s="15" t="n"/>
@@ -4731,7 +4731,7 @@
       </c>
       <c r="W50" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X50" s="15" t="n"/>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="W51" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X51" s="15" t="n"/>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="W52" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X52" s="15" t="n"/>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="W53" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X53" s="15" t="n"/>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="W54" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Manual list</t>
         </is>
       </c>
       <c r="X54" s="15" t="n"/>
@@ -6788,7 +6788,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="W6:W72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not started,Pilot,Discovering,Discovered,Imported,Live,Excluded"</formula1>
+      <formula1>"Not started,Manual list,Discovering,Discovered,Imported,Live,Excluded"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>4903</v>
+        <v>3986</v>
       </c>
     </row>
   </sheetData>
@@ -6972,7 +6972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7006,38 +7006,56 @@
     <row r="2">
       <c r="A2" s="21" t="inlineStr">
         <is>
+          <t>full-uae</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="n">
+        <v>917</v>
+      </c>
+      <c r="D2" s="21" t="n">
+        <v>10776</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
           <t>pilot-dubai</t>
         </is>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="C2" s="21" t="n">
+      <c r="C3" s="21" t="n">
         <v>97</v>
       </c>
-      <c r="D2" s="21" t="n">
+      <c r="D3" s="21" t="n">
         <v>1621</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C3" s="25">
-        <f>SUM(C2:C2)</f>
-        <v/>
-      </c>
-      <c r="D3" s="25">
-        <f>SUM(D2:D2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="C4" s="25">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+      <c r="D4" s="25">
+        <f>SUM(D2:D3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Unique places per run; the Tracker deduplicates across runs, so its total can be lower.</t>
         </is>

</xml_diff>

<commit_message>
Tracker: discovery batch 2 (2,014 searches, 21,244 unique places)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reviewencer-data-tracker.xlsx
+++ b/docs/Reviewencer-data-tracker.xlsx
@@ -331,7 +331,7 @@
     </comment>
     <comment ref="B18" authorId="0" shapeId="0">
       <text>
-        <t>Read from the SerpAPI account page at 2026-10-21 11:52 (free lookup). Refreshes when the tracker is regenerated.</t>
+        <t>Read from the SerpAPI account page at 2026-10-21 14:05 (free lookup). Refreshes when the tracker is regenerated.</t>
       </text>
     </comment>
   </commentList>
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-21 11:52 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
+          <t>Generated 2026-10-21 14:05 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
         </is>
       </c>
     </row>
@@ -1312,25 +1312,25 @@
         <v>0</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P11" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="S11" s="12" t="n">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="T11" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="U11" s="12" t="n">
-        <v>0</v>
+        <v>177</v>
       </c>
       <c r="V11" s="13">
         <f>IFERROR(SUM(Q11:U11)/(5*P11),0)</f>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="W11" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X11" s="15" t="n"/>
@@ -1747,25 +1747,25 @@
         <v>0</v>
       </c>
       <c r="O16" s="12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P16" s="12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="Q16" s="12" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="R16" s="12" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="S16" s="12" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="T16" s="12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="U16" s="12" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="V16" s="13">
         <f>IFERROR(SUM(Q16:U16)/(5*P16),0)</f>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="W16" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X16" s="15" t="n"/>
@@ -1921,25 +1921,25 @@
         <v>0</v>
       </c>
       <c r="O18" s="12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P18" s="12" t="n">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="Q18" s="12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="R18" s="12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="S18" s="12" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="T18" s="12" t="n">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="U18" s="12" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="V18" s="13">
         <f>IFERROR(SUM(Q18:U18)/(5*P18),0)</f>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="W18" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X18" s="15" t="n"/>
@@ -2008,25 +2008,25 @@
         <v>0</v>
       </c>
       <c r="O19" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P19" s="12" t="n">
-        <v>0</v>
+        <v>766</v>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>0</v>
+        <v>676</v>
       </c>
       <c r="R19" s="12" t="n">
-        <v>0</v>
+        <v>756</v>
       </c>
       <c r="S19" s="12" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="T19" s="12" t="n">
-        <v>0</v>
+        <v>766</v>
       </c>
       <c r="U19" s="12" t="n">
-        <v>0</v>
+        <v>681</v>
       </c>
       <c r="V19" s="13">
         <f>IFERROR(SUM(Q19:U19)/(5*P19),0)</f>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="W19" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X19" s="15" t="n"/>
@@ -2095,25 +2095,25 @@
         <v>0</v>
       </c>
       <c r="O20" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P20" s="12" t="n">
-        <v>0</v>
+        <v>598</v>
       </c>
       <c r="Q20" s="12" t="n">
-        <v>0</v>
+        <v>522</v>
       </c>
       <c r="R20" s="12" t="n">
-        <v>0</v>
+        <v>585</v>
       </c>
       <c r="S20" s="12" t="n">
-        <v>0</v>
+        <v>582</v>
       </c>
       <c r="T20" s="12" t="n">
-        <v>0</v>
+        <v>598</v>
       </c>
       <c r="U20" s="12" t="n">
-        <v>0</v>
+        <v>524</v>
       </c>
       <c r="V20" s="13">
         <f>IFERROR(SUM(Q20:U20)/(5*P20),0)</f>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="W20" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X20" s="15" t="n"/>
@@ -2356,25 +2356,25 @@
         <v>0</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="P23" s="12" t="n">
-        <v>224</v>
+        <v>518</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>184</v>
+        <v>379</v>
       </c>
       <c r="R23" s="12" t="n">
-        <v>219</v>
+        <v>510</v>
       </c>
       <c r="S23" s="12" t="n">
-        <v>221</v>
+        <v>508</v>
       </c>
       <c r="T23" s="12" t="n">
-        <v>224</v>
+        <v>518</v>
       </c>
       <c r="U23" s="12" t="n">
-        <v>183</v>
+        <v>392</v>
       </c>
       <c r="V23" s="13">
         <f>IFERROR(SUM(Q23:U23)/(5*P23),0)</f>
@@ -2530,25 +2530,25 @@
         <v>0</v>
       </c>
       <c r="O25" s="12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P25" s="12" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="Q25" s="12" t="n">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="R25" s="12" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="S25" s="12" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="T25" s="12" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="U25" s="12" t="n">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="V25" s="13">
         <f>IFERROR(SUM(Q25:U25)/(5*P25),0)</f>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="W25" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X25" s="15" t="n"/>
@@ -2617,25 +2617,25 @@
         <v>0</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P26" s="12" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="R26" s="12" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="S26" s="12" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="T26" s="12" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="U26" s="12" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="V26" s="13">
         <f>IFERROR(SUM(Q26:U26)/(5*P26),0)</f>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="W26" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X26" s="15" t="n"/>
@@ -2704,25 +2704,25 @@
         <v>0</v>
       </c>
       <c r="O27" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P27" s="12" t="n">
-        <v>0</v>
+        <v>376</v>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>0</v>
+        <v>351</v>
       </c>
       <c r="R27" s="12" t="n">
-        <v>0</v>
+        <v>366</v>
       </c>
       <c r="S27" s="12" t="n">
-        <v>0</v>
+        <v>359</v>
       </c>
       <c r="T27" s="12" t="n">
-        <v>0</v>
+        <v>376</v>
       </c>
       <c r="U27" s="12" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="V27" s="13">
         <f>IFERROR(SUM(Q27:U27)/(5*P27),0)</f>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="W27" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X27" s="15" t="n"/>
@@ -2791,25 +2791,25 @@
         <v>0</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P28" s="12" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>0</v>
+        <v>454</v>
       </c>
       <c r="R28" s="12" t="n">
-        <v>0</v>
+        <v>519</v>
       </c>
       <c r="S28" s="12" t="n">
-        <v>0</v>
+        <v>511</v>
       </c>
       <c r="T28" s="12" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="U28" s="12" t="n">
-        <v>0</v>
+        <v>385</v>
       </c>
       <c r="V28" s="13">
         <f>IFERROR(SUM(Q28:U28)/(5*P28),0)</f>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="W28" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X28" s="15" t="n"/>
@@ -2878,25 +2878,25 @@
         <v>0</v>
       </c>
       <c r="O29" s="12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P29" s="12" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="Q29" s="12" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="R29" s="12" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="S29" s="12" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="T29" s="12" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="U29" s="12" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="V29" s="13">
         <f>IFERROR(SUM(Q29:U29)/(5*P29),0)</f>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="W29" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X29" s="15" t="n"/>
@@ -2965,25 +2965,25 @@
         <v>0</v>
       </c>
       <c r="O30" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P30" s="12" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
       <c r="Q30" s="12" t="n">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="R30" s="12" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="S30" s="12" t="n">
-        <v>0</v>
+        <v>351</v>
       </c>
       <c r="T30" s="12" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
       <c r="U30" s="12" t="n">
-        <v>0</v>
+        <v>272</v>
       </c>
       <c r="V30" s="13">
         <f>IFERROR(SUM(Q30:U30)/(5*P30),0)</f>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="W30" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X30" s="15" t="n"/>
@@ -3052,25 +3052,25 @@
         <v>0</v>
       </c>
       <c r="O31" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P31" s="12" t="n">
-        <v>0</v>
+        <v>226</v>
       </c>
       <c r="Q31" s="12" t="n">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="R31" s="12" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="S31" s="12" t="n">
-        <v>0</v>
+        <v>217</v>
       </c>
       <c r="T31" s="12" t="n">
-        <v>0</v>
+        <v>226</v>
       </c>
       <c r="U31" s="12" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="V31" s="13">
         <f>IFERROR(SUM(Q31:U31)/(5*P31),0)</f>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="W31" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X31" s="15" t="n"/>
@@ -3139,25 +3139,25 @@
         <v>0</v>
       </c>
       <c r="O32" s="12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P32" s="12" t="n">
-        <v>0</v>
+        <v>177</v>
       </c>
       <c r="Q32" s="12" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="R32" s="12" t="n">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="S32" s="12" t="n">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="T32" s="12" t="n">
-        <v>0</v>
+        <v>177</v>
       </c>
       <c r="U32" s="12" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="V32" s="13">
         <f>IFERROR(SUM(Q32:U32)/(5*P32),0)</f>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="W32" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X32" s="15" t="n"/>
@@ -3226,25 +3226,25 @@
         <v>0</v>
       </c>
       <c r="O33" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P33" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="Q33" s="12" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="R33" s="12" t="n">
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="S33" s="12" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="T33" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="U33" s="12" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="V33" s="13">
         <f>IFERROR(SUM(Q33:U33)/(5*P33),0)</f>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="W33" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X33" s="15" t="n"/>
@@ -3313,25 +3313,25 @@
         <v>0</v>
       </c>
       <c r="O34" s="12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P34" s="12" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="Q34" s="12" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="R34" s="12" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="S34" s="12" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="T34" s="12" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="U34" s="12" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="V34" s="13">
         <f>IFERROR(SUM(Q34:U34)/(5*P34),0)</f>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="W34" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X34" s="15" t="n"/>
@@ -3400,25 +3400,25 @@
         <v>0</v>
       </c>
       <c r="O35" s="12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P35" s="12" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="Q35" s="12" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="R35" s="12" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="S35" s="12" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="T35" s="12" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="U35" s="12" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="V35" s="13">
         <f>IFERROR(SUM(Q35:U35)/(5*P35),0)</f>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="W35" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X35" s="15" t="n"/>
@@ -3487,25 +3487,25 @@
         <v>0</v>
       </c>
       <c r="O36" s="12" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P36" s="12" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="Q36" s="12" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="R36" s="12" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="S36" s="12" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="T36" s="12" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="U36" s="12" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="V36" s="13">
         <f>IFERROR(SUM(Q36:U36)/(5*P36),0)</f>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="W36" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X36" s="15" t="n"/>
@@ -3661,25 +3661,25 @@
         <v>0</v>
       </c>
       <c r="O38" s="12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P38" s="12" t="n">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="Q38" s="12" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="R38" s="12" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="S38" s="12" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="T38" s="12" t="n">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="U38" s="12" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="V38" s="13">
         <f>IFERROR(SUM(Q38:U38)/(5*P38),0)</f>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="W38" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X38" s="15" t="n"/>
@@ -3748,25 +3748,25 @@
         <v>0</v>
       </c>
       <c r="O39" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P39" s="12" t="n">
-        <v>0</v>
+        <v>562</v>
       </c>
       <c r="Q39" s="12" t="n">
-        <v>0</v>
+        <v>465</v>
       </c>
       <c r="R39" s="12" t="n">
-        <v>0</v>
+        <v>506</v>
       </c>
       <c r="S39" s="12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T39" s="12" t="n">
-        <v>0</v>
+        <v>562</v>
       </c>
       <c r="U39" s="12" t="n">
-        <v>0</v>
+        <v>468</v>
       </c>
       <c r="V39" s="13">
         <f>IFERROR(SUM(Q39:U39)/(5*P39),0)</f>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="W39" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X39" s="15" t="n"/>
@@ -3835,25 +3835,25 @@
         <v>0</v>
       </c>
       <c r="O40" s="12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P40" s="12" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="Q40" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="R40" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="S40" s="12" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="T40" s="12" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="U40" s="12" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="V40" s="13">
         <f>IFERROR(SUM(Q40:U40)/(5*P40),0)</f>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="W40" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X40" s="15" t="n"/>
@@ -3922,25 +3922,25 @@
         <v>0</v>
       </c>
       <c r="O41" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P41" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="Q41" s="12" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="R41" s="12" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="S41" s="12" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="T41" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="U41" s="12" t="n">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="V41" s="13">
         <f>IFERROR(SUM(Q41:U41)/(5*P41),0)</f>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="W41" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X41" s="15" t="n"/>
@@ -4009,25 +4009,25 @@
         <v>0</v>
       </c>
       <c r="O42" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P42" s="12" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="Q42" s="12" t="n">
-        <v>0</v>
+        <v>214</v>
       </c>
       <c r="R42" s="12" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="S42" s="12" t="n">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="T42" s="12" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="U42" s="12" t="n">
-        <v>0</v>
+        <v>211</v>
       </c>
       <c r="V42" s="13">
         <f>IFERROR(SUM(Q42:U42)/(5*P42),0)</f>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="W42" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X42" s="15" t="n"/>
@@ -4183,25 +4183,25 @@
         <v>0</v>
       </c>
       <c r="O44" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P44" s="12" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="Q44" s="12" t="n">
-        <v>0</v>
+        <v>206</v>
       </c>
       <c r="R44" s="12" t="n">
-        <v>0</v>
+        <v>233</v>
       </c>
       <c r="S44" s="12" t="n">
-        <v>0</v>
+        <v>234</v>
       </c>
       <c r="T44" s="12" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="U44" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="V44" s="13">
         <f>IFERROR(SUM(Q44:U44)/(5*P44),0)</f>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="W44" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X44" s="15" t="n"/>
@@ -4270,25 +4270,25 @@
         <v>0</v>
       </c>
       <c r="O45" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P45" s="12" t="n">
-        <v>0</v>
+        <v>488</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>0</v>
+        <v>364</v>
       </c>
       <c r="R45" s="12" t="n">
-        <v>0</v>
+        <v>476</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>0</v>
+        <v>483</v>
       </c>
       <c r="T45" s="12" t="n">
-        <v>0</v>
+        <v>488</v>
       </c>
       <c r="U45" s="12" t="n">
-        <v>0</v>
+        <v>371</v>
       </c>
       <c r="V45" s="13">
         <f>IFERROR(SUM(Q45:U45)/(5*P45),0)</f>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="W45" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X45" s="15" t="n"/>
@@ -4357,25 +4357,25 @@
         <v>0</v>
       </c>
       <c r="O46" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P46" s="12" t="n">
-        <v>0</v>
+        <v>453</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>0</v>
+        <v>274</v>
       </c>
       <c r="R46" s="12" t="n">
-        <v>0</v>
+        <v>407</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>0</v>
+        <v>425</v>
       </c>
       <c r="T46" s="12" t="n">
-        <v>0</v>
+        <v>453</v>
       </c>
       <c r="U46" s="12" t="n">
-        <v>0</v>
+        <v>293</v>
       </c>
       <c r="V46" s="13">
         <f>IFERROR(SUM(Q46:U46)/(5*P46),0)</f>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="W46" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X46" s="15" t="n"/>
@@ -4444,25 +4444,25 @@
         <v>0</v>
       </c>
       <c r="O47" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P47" s="12" t="n">
-        <v>0</v>
+        <v>234</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="R47" s="12" t="n">
-        <v>0</v>
+        <v>231</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>0</v>
+        <v>231</v>
       </c>
       <c r="T47" s="12" t="n">
-        <v>0</v>
+        <v>234</v>
       </c>
       <c r="U47" s="12" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="V47" s="13">
         <f>IFERROR(SUM(Q47:U47)/(5*P47),0)</f>
@@ -4470,7 +4470,7 @@
       </c>
       <c r="W47" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X47" s="15" t="n"/>
@@ -4531,25 +4531,25 @@
         <v>0</v>
       </c>
       <c r="O48" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P48" s="12" t="n">
-        <v>0</v>
+        <v>231</v>
       </c>
       <c r="Q48" s="12" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="R48" s="12" t="n">
-        <v>0</v>
+        <v>228</v>
       </c>
       <c r="S48" s="12" t="n">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="T48" s="12" t="n">
-        <v>0</v>
+        <v>231</v>
       </c>
       <c r="U48" s="12" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="V48" s="13">
         <f>IFERROR(SUM(Q48:U48)/(5*P48),0)</f>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="W48" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X48" s="15" t="n"/>
@@ -5140,25 +5140,25 @@
         <v>0</v>
       </c>
       <c r="O55" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P55" s="12" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="Q55" s="12" t="n">
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="R55" s="12" t="n">
-        <v>0</v>
+        <v>521</v>
       </c>
       <c r="S55" s="12" t="n">
-        <v>0</v>
+        <v>519</v>
       </c>
       <c r="T55" s="12" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="U55" s="12" t="n">
-        <v>0</v>
+        <v>351</v>
       </c>
       <c r="V55" s="13">
         <f>IFERROR(SUM(Q55:U55)/(5*P55),0)</f>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="W55" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X55" s="15" t="n"/>
@@ -5227,25 +5227,25 @@
         <v>0</v>
       </c>
       <c r="O56" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P56" s="12" t="n">
-        <v>0</v>
+        <v>790</v>
       </c>
       <c r="Q56" s="12" t="n">
-        <v>0</v>
+        <v>570</v>
       </c>
       <c r="R56" s="12" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="S56" s="12" t="n">
-        <v>0</v>
+        <v>776</v>
       </c>
       <c r="T56" s="12" t="n">
-        <v>0</v>
+        <v>790</v>
       </c>
       <c r="U56" s="12" t="n">
-        <v>0</v>
+        <v>526</v>
       </c>
       <c r="V56" s="13">
         <f>IFERROR(SUM(Q56:U56)/(5*P56),0)</f>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="W56" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X56" s="15" t="n"/>
@@ -5314,25 +5314,25 @@
         <v>0</v>
       </c>
       <c r="O57" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P57" s="12" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="Q57" s="12" t="n">
-        <v>0</v>
+        <v>206</v>
       </c>
       <c r="R57" s="12" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="S57" s="12" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="T57" s="12" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="U57" s="12" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="V57" s="13">
         <f>IFERROR(SUM(Q57:U57)/(5*P57),0)</f>
@@ -5340,7 +5340,7 @@
       </c>
       <c r="W57" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X57" s="15" t="n"/>
@@ -5401,25 +5401,25 @@
         <v>0</v>
       </c>
       <c r="O58" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P58" s="12" t="n">
-        <v>0</v>
+        <v>528</v>
       </c>
       <c r="Q58" s="12" t="n">
-        <v>0</v>
+        <v>375</v>
       </c>
       <c r="R58" s="12" t="n">
-        <v>0</v>
+        <v>516</v>
       </c>
       <c r="S58" s="12" t="n">
-        <v>0</v>
+        <v>522</v>
       </c>
       <c r="T58" s="12" t="n">
-        <v>0</v>
+        <v>528</v>
       </c>
       <c r="U58" s="12" t="n">
-        <v>0</v>
+        <v>401</v>
       </c>
       <c r="V58" s="13">
         <f>IFERROR(SUM(Q58:U58)/(5*P58),0)</f>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="W58" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X58" s="15" t="n"/>
@@ -5488,25 +5488,25 @@
         <v>0</v>
       </c>
       <c r="O59" s="12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P59" s="12" t="n">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="Q59" s="12" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="R59" s="12" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="S59" s="12" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="T59" s="12" t="n">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="U59" s="12" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="V59" s="13">
         <f>IFERROR(SUM(Q59:U59)/(5*P59),0)</f>
@@ -5514,7 +5514,7 @@
       </c>
       <c r="W59" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X59" s="15" t="n"/>
@@ -5575,25 +5575,25 @@
         <v>0</v>
       </c>
       <c r="O60" s="12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P60" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="Q60" s="12" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="R60" s="12" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="S60" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="T60" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="U60" s="12" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="V60" s="13">
         <f>IFERROR(SUM(Q60:U60)/(5*P60),0)</f>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="W60" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X60" s="15" t="n"/>
@@ -5923,25 +5923,25 @@
         <v>0</v>
       </c>
       <c r="O64" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P64" s="12" t="n">
-        <v>0</v>
+        <v>538</v>
       </c>
       <c r="Q64" s="12" t="n">
-        <v>0</v>
+        <v>404</v>
       </c>
       <c r="R64" s="12" t="n">
-        <v>0</v>
+        <v>524</v>
       </c>
       <c r="S64" s="12" t="n">
-        <v>0</v>
+        <v>531</v>
       </c>
       <c r="T64" s="12" t="n">
-        <v>0</v>
+        <v>538</v>
       </c>
       <c r="U64" s="12" t="n">
-        <v>0</v>
+        <v>372</v>
       </c>
       <c r="V64" s="13">
         <f>IFERROR(SUM(Q64:U64)/(5*P64),0)</f>
@@ -5949,7 +5949,7 @@
       </c>
       <c r="W64" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X64" s="15" t="n"/>
@@ -6097,25 +6097,25 @@
         <v>0</v>
       </c>
       <c r="O66" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P66" s="12" t="n">
-        <v>0</v>
+        <v>538</v>
       </c>
       <c r="Q66" s="12" t="n">
-        <v>0</v>
+        <v>282</v>
       </c>
       <c r="R66" s="12" t="n">
-        <v>0</v>
+        <v>526</v>
       </c>
       <c r="S66" s="12" t="n">
-        <v>0</v>
+        <v>531</v>
       </c>
       <c r="T66" s="12" t="n">
-        <v>0</v>
+        <v>538</v>
       </c>
       <c r="U66" s="12" t="n">
-        <v>0</v>
+        <v>318</v>
       </c>
       <c r="V66" s="13">
         <f>IFERROR(SUM(Q66:U66)/(5*P66),0)</f>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="W66" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X66" s="15" t="n"/>
@@ -6184,25 +6184,25 @@
         <v>0</v>
       </c>
       <c r="O67" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P67" s="12" t="n">
-        <v>0</v>
+        <v>234</v>
       </c>
       <c r="Q67" s="12" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="R67" s="12" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="S67" s="12" t="n">
-        <v>0</v>
+        <v>229</v>
       </c>
       <c r="T67" s="12" t="n">
-        <v>0</v>
+        <v>234</v>
       </c>
       <c r="U67" s="12" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="V67" s="13">
         <f>IFERROR(SUM(Q67:U67)/(5*P67),0)</f>
@@ -6210,7 +6210,7 @@
       </c>
       <c r="W67" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X67" s="15" t="n"/>
@@ -6271,25 +6271,25 @@
         <v>0</v>
       </c>
       <c r="O68" s="12" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P68" s="12" t="n">
-        <v>0</v>
+        <v>364</v>
       </c>
       <c r="Q68" s="12" t="n">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="R68" s="12" t="n">
-        <v>0</v>
+        <v>353</v>
       </c>
       <c r="S68" s="12" t="n">
-        <v>0</v>
+        <v>357</v>
       </c>
       <c r="T68" s="12" t="n">
-        <v>0</v>
+        <v>364</v>
       </c>
       <c r="U68" s="12" t="n">
-        <v>0</v>
+        <v>266</v>
       </c>
       <c r="V68" s="13">
         <f>IFERROR(SUM(Q68:U68)/(5*P68),0)</f>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="W68" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X68" s="15" t="n"/>
@@ -6358,25 +6358,25 @@
         <v>0</v>
       </c>
       <c r="O69" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P69" s="12" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="Q69" s="12" t="n">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="R69" s="12" t="n">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="S69" s="12" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="T69" s="12" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="U69" s="12" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="V69" s="13">
         <f>IFERROR(SUM(Q69:U69)/(5*P69),0)</f>
@@ -6384,7 +6384,7 @@
       </c>
       <c r="W69" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X69" s="15" t="n"/>
@@ -6445,25 +6445,25 @@
         <v>0</v>
       </c>
       <c r="O70" s="12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P70" s="12" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="Q70" s="12" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="R70" s="12" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="S70" s="12" t="n">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="T70" s="12" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="U70" s="12" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="V70" s="13">
         <f>IFERROR(SUM(Q70:U70)/(5*P70),0)</f>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="W70" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X70" s="15" t="n"/>
@@ -6532,25 +6532,25 @@
         <v>0</v>
       </c>
       <c r="O71" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P71" s="12" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="Q71" s="12" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="R71" s="12" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="S71" s="12" t="n">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="T71" s="12" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="U71" s="12" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="V71" s="13">
         <f>IFERROR(SUM(Q71:U71)/(5*P71),0)</f>
@@ -6558,7 +6558,7 @@
       </c>
       <c r="W71" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X71" s="15" t="n"/>
@@ -6619,25 +6619,25 @@
         <v>0</v>
       </c>
       <c r="O72" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P72" s="12" t="n">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="Q72" s="12" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="R72" s="12" t="n">
-        <v>0</v>
+        <v>218</v>
       </c>
       <c r="S72" s="12" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="T72" s="12" t="n">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="U72" s="12" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="V72" s="13">
         <f>IFERROR(SUM(Q72:U72)/(5*P72),0)</f>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="W72" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X72" s="15" t="n"/>
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>3986</v>
+        <v>2986</v>
       </c>
     </row>
   </sheetData>
@@ -7015,10 +7015,10 @@
         </is>
       </c>
       <c r="C2" s="21" t="n">
-        <v>917</v>
+        <v>1917</v>
       </c>
       <c r="D2" s="21" t="n">
-        <v>10776</v>
+        <v>21244</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Discovery batch 3: Northern Emirates, extra areas, chains
- serp-discovery.ts: shared DENSE/COMMON category lists; new runs
  northern-emirates (Ajman, RAK, Fujairah, UAQ), more-areas (13 Dubai +
  3 Sharjah neighbourhoods) and chains (70 chains with 4+ locations,
  searched per main city; files prefixed <category>~<chain>).
- data_tracker.py: counts chain files under their category.
- Tracker: 2,938 searches total, 30,612 unique businesses across all 7
  emirates, all 60 map categories discovered.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reviewencer-data-tracker.xlsx
+++ b/docs/Reviewencer-data-tracker.xlsx
@@ -331,7 +331,7 @@
     </comment>
     <comment ref="B18" authorId="0" shapeId="0">
       <text>
-        <t>Read from the SerpAPI account page at 2026-10-21 14:05 (free lookup). Refreshes when the tracker is regenerated.</t>
+        <t>Read from the SerpAPI account page at 2026-10-21 19:43 (free lookup). Refreshes when the tracker is regenerated.</t>
       </text>
     </comment>
   </commentList>
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-21 14:05 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
+          <t>Generated 2026-10-21 19:43 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
         </is>
       </c>
     </row>
@@ -877,25 +877,25 @@
         <v>0</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>2121</v>
+        <v>2487</v>
       </c>
       <c r="Q6" s="12" t="n">
-        <v>1552</v>
+        <v>1781</v>
       </c>
       <c r="R6" s="12" t="n">
-        <v>2078</v>
+        <v>2432</v>
       </c>
       <c r="S6" s="12" t="n">
-        <v>2091</v>
+        <v>2452</v>
       </c>
       <c r="T6" s="12" t="n">
-        <v>2121</v>
+        <v>2487</v>
       </c>
       <c r="U6" s="12" t="n">
-        <v>2065</v>
+        <v>2420</v>
       </c>
       <c r="V6" s="13">
         <f>IFERROR(SUM(Q6:U6)/(5*P6),0)</f>
@@ -964,25 +964,25 @@
         <v>0</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>102</v>
+        <v>144</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>1740</v>
+        <v>2349</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>1241</v>
+        <v>1669</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>1654</v>
+        <v>2222</v>
       </c>
       <c r="S7" s="12" t="n">
-        <v>1695</v>
+        <v>2296</v>
       </c>
       <c r="T7" s="12" t="n">
-        <v>1740</v>
+        <v>2349</v>
       </c>
       <c r="U7" s="12" t="n">
-        <v>1592</v>
+        <v>2140</v>
       </c>
       <c r="V7" s="13">
         <f>IFERROR(SUM(Q7:U7)/(5*P7),0)</f>
@@ -1051,25 +1051,25 @@
         <v>0</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>900</v>
+        <v>1358</v>
       </c>
       <c r="Q8" s="12" t="n">
-        <v>679</v>
+        <v>968</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>880</v>
+        <v>1330</v>
       </c>
       <c r="S8" s="12" t="n">
-        <v>892</v>
+        <v>1344</v>
       </c>
       <c r="T8" s="12" t="n">
-        <v>900</v>
+        <v>1358</v>
       </c>
       <c r="U8" s="12" t="n">
-        <v>877</v>
+        <v>1321</v>
       </c>
       <c r="V8" s="13">
         <f>IFERROR(SUM(Q8:U8)/(5*P8),0)</f>
@@ -1138,25 +1138,25 @@
         <v>0</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>729</v>
+        <v>1099</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>534</v>
+        <v>730</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>702</v>
+        <v>1056</v>
       </c>
       <c r="S9" s="12" t="n">
-        <v>717</v>
+        <v>1076</v>
       </c>
       <c r="T9" s="12" t="n">
-        <v>729</v>
+        <v>1099</v>
       </c>
       <c r="U9" s="12" t="n">
-        <v>646</v>
+        <v>942</v>
       </c>
       <c r="V9" s="13">
         <f>IFERROR(SUM(Q9:U9)/(5*P9),0)</f>
@@ -1225,25 +1225,25 @@
         <v>0</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="P10" s="12" t="n">
-        <v>809</v>
+        <v>1195</v>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>616</v>
+        <v>855</v>
       </c>
       <c r="R10" s="12" t="n">
-        <v>776</v>
+        <v>1148</v>
       </c>
       <c r="S10" s="12" t="n">
-        <v>800</v>
+        <v>1179</v>
       </c>
       <c r="T10" s="12" t="n">
-        <v>809</v>
+        <v>1195</v>
       </c>
       <c r="U10" s="12" t="n">
-        <v>742</v>
+        <v>1072</v>
       </c>
       <c r="V10" s="13">
         <f>IFERROR(SUM(Q10:U10)/(5*P10),0)</f>
@@ -1399,25 +1399,25 @@
         <v>0</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P12" s="12" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="Q12" s="12" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="R12" s="12" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="S12" s="12" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="T12" s="12" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="U12" s="12" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="V12" s="13">
         <f>IFERROR(SUM(Q12:U12)/(5*P12),0)</f>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="W12" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X12" s="15" t="n"/>
@@ -1486,25 +1486,25 @@
         <v>0</v>
       </c>
       <c r="O13" s="12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P13" s="12" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="Q13" s="12" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="R13" s="12" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="S13" s="12" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="T13" s="12" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="U13" s="12" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="V13" s="13">
         <f>IFERROR(SUM(Q13:U13)/(5*P13),0)</f>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="W13" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X13" s="15" t="n"/>
@@ -1573,25 +1573,25 @@
         <v>0</v>
       </c>
       <c r="O14" s="12" t="n">
-        <v>51</v>
+        <v>102</v>
       </c>
       <c r="P14" s="12" t="n">
-        <v>817</v>
+        <v>1419</v>
       </c>
       <c r="Q14" s="12" t="n">
-        <v>504</v>
+        <v>896</v>
       </c>
       <c r="R14" s="12" t="n">
-        <v>776</v>
+        <v>1348</v>
       </c>
       <c r="S14" s="12" t="n">
-        <v>800</v>
+        <v>1388</v>
       </c>
       <c r="T14" s="12" t="n">
-        <v>817</v>
+        <v>1419</v>
       </c>
       <c r="U14" s="12" t="n">
-        <v>709</v>
+        <v>1218</v>
       </c>
       <c r="V14" s="13">
         <f>IFERROR(SUM(Q14:U14)/(5*P14),0)</f>
@@ -1660,25 +1660,25 @@
         <v>0</v>
       </c>
       <c r="O15" s="12" t="n">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="P15" s="12" t="n">
-        <v>517</v>
+        <v>742</v>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>301</v>
+        <v>402</v>
       </c>
       <c r="R15" s="12" t="n">
-        <v>470</v>
+        <v>669</v>
       </c>
       <c r="S15" s="12" t="n">
-        <v>504</v>
+        <v>717</v>
       </c>
       <c r="T15" s="12" t="n">
-        <v>517</v>
+        <v>742</v>
       </c>
       <c r="U15" s="12" t="n">
-        <v>404</v>
+        <v>543</v>
       </c>
       <c r="V15" s="13">
         <f>IFERROR(SUM(Q15:U15)/(5*P15),0)</f>
@@ -1834,25 +1834,25 @@
         <v>0</v>
       </c>
       <c r="O17" s="12" t="n">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="P17" s="12" t="n">
-        <v>1375</v>
+        <v>1754</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>1137</v>
+        <v>1432</v>
       </c>
       <c r="R17" s="12" t="n">
-        <v>1325</v>
+        <v>1693</v>
       </c>
       <c r="S17" s="12" t="n">
-        <v>1308</v>
+        <v>1681</v>
       </c>
       <c r="T17" s="12" t="n">
-        <v>1375</v>
+        <v>1754</v>
       </c>
       <c r="U17" s="12" t="n">
-        <v>1123</v>
+        <v>1443</v>
       </c>
       <c r="V17" s="13">
         <f>IFERROR(SUM(Q17:U17)/(5*P17),0)</f>
@@ -2008,25 +2008,25 @@
         <v>0</v>
       </c>
       <c r="O19" s="12" t="n">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="P19" s="12" t="n">
-        <v>766</v>
+        <v>1131</v>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>676</v>
+        <v>971</v>
       </c>
       <c r="R19" s="12" t="n">
-        <v>756</v>
+        <v>1118</v>
       </c>
       <c r="S19" s="12" t="n">
-        <v>750</v>
+        <v>1108</v>
       </c>
       <c r="T19" s="12" t="n">
-        <v>766</v>
+        <v>1131</v>
       </c>
       <c r="U19" s="12" t="n">
-        <v>681</v>
+        <v>1008</v>
       </c>
       <c r="V19" s="13">
         <f>IFERROR(SUM(Q19:U19)/(5*P19),0)</f>
@@ -2095,25 +2095,25 @@
         <v>0</v>
       </c>
       <c r="O20" s="12" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="P20" s="12" t="n">
-        <v>598</v>
+        <v>899</v>
       </c>
       <c r="Q20" s="12" t="n">
-        <v>522</v>
+        <v>746</v>
       </c>
       <c r="R20" s="12" t="n">
-        <v>585</v>
+        <v>881</v>
       </c>
       <c r="S20" s="12" t="n">
-        <v>582</v>
+        <v>880</v>
       </c>
       <c r="T20" s="12" t="n">
-        <v>598</v>
+        <v>899</v>
       </c>
       <c r="U20" s="12" t="n">
-        <v>524</v>
+        <v>780</v>
       </c>
       <c r="V20" s="13">
         <f>IFERROR(SUM(Q20:U20)/(5*P20),0)</f>
@@ -2182,25 +2182,25 @@
         <v>0</v>
       </c>
       <c r="O21" s="12" t="n">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="P21" s="12" t="n">
-        <v>1144</v>
+        <v>1377</v>
       </c>
       <c r="Q21" s="12" t="n">
-        <v>965</v>
+        <v>1119</v>
       </c>
       <c r="R21" s="12" t="n">
-        <v>1130</v>
+        <v>1359</v>
       </c>
       <c r="S21" s="12" t="n">
-        <v>1124</v>
+        <v>1353</v>
       </c>
       <c r="T21" s="12" t="n">
-        <v>1144</v>
+        <v>1377</v>
       </c>
       <c r="U21" s="12" t="n">
-        <v>969</v>
+        <v>1166</v>
       </c>
       <c r="V21" s="13">
         <f>IFERROR(SUM(Q21:U21)/(5*P21),0)</f>
@@ -2269,25 +2269,25 @@
         <v>0</v>
       </c>
       <c r="O22" s="12" t="n">
-        <v>51</v>
+        <v>102</v>
       </c>
       <c r="P22" s="12" t="n">
-        <v>760</v>
+        <v>1344</v>
       </c>
       <c r="Q22" s="12" t="n">
-        <v>643</v>
+        <v>1081</v>
       </c>
       <c r="R22" s="12" t="n">
-        <v>750</v>
+        <v>1325</v>
       </c>
       <c r="S22" s="12" t="n">
-        <v>749</v>
+        <v>1324</v>
       </c>
       <c r="T22" s="12" t="n">
-        <v>760</v>
+        <v>1344</v>
       </c>
       <c r="U22" s="12" t="n">
-        <v>615</v>
+        <v>1026</v>
       </c>
       <c r="V22" s="13">
         <f>IFERROR(SUM(Q22:U22)/(5*P22),0)</f>
@@ -2356,25 +2356,25 @@
         <v>0</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="P23" s="12" t="n">
-        <v>518</v>
+        <v>854</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>379</v>
+        <v>586</v>
       </c>
       <c r="R23" s="12" t="n">
-        <v>510</v>
+        <v>841</v>
       </c>
       <c r="S23" s="12" t="n">
-        <v>508</v>
+        <v>833</v>
       </c>
       <c r="T23" s="12" t="n">
-        <v>518</v>
+        <v>854</v>
       </c>
       <c r="U23" s="12" t="n">
-        <v>392</v>
+        <v>600</v>
       </c>
       <c r="V23" s="13">
         <f>IFERROR(SUM(Q23:U23)/(5*P23),0)</f>
@@ -2443,25 +2443,25 @@
         <v>0</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="P24" s="12" t="n">
-        <v>1506</v>
+        <v>1878</v>
       </c>
       <c r="Q24" s="12" t="n">
-        <v>1099</v>
+        <v>1351</v>
       </c>
       <c r="R24" s="12" t="n">
-        <v>1440</v>
+        <v>1806</v>
       </c>
       <c r="S24" s="12" t="n">
-        <v>1483</v>
+        <v>1853</v>
       </c>
       <c r="T24" s="12" t="n">
-        <v>1506</v>
+        <v>1878</v>
       </c>
       <c r="U24" s="12" t="n">
-        <v>1308</v>
+        <v>1630</v>
       </c>
       <c r="V24" s="13">
         <f>IFERROR(SUM(Q24:U24)/(5*P24),0)</f>
@@ -2617,25 +2617,25 @@
         <v>0</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P26" s="12" t="n">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="R26" s="12" t="n">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="S26" s="12" t="n">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="T26" s="12" t="n">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="U26" s="12" t="n">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="V26" s="13">
         <f>IFERROR(SUM(Q26:U26)/(5*P26),0)</f>
@@ -2704,25 +2704,25 @@
         <v>0</v>
       </c>
       <c r="O27" s="12" t="n">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="P27" s="12" t="n">
-        <v>376</v>
+        <v>527</v>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>351</v>
+        <v>470</v>
       </c>
       <c r="R27" s="12" t="n">
-        <v>366</v>
+        <v>510</v>
       </c>
       <c r="S27" s="12" t="n">
-        <v>359</v>
+        <v>492</v>
       </c>
       <c r="T27" s="12" t="n">
-        <v>376</v>
+        <v>527</v>
       </c>
       <c r="U27" s="12" t="n">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="V27" s="13">
         <f>IFERROR(SUM(Q27:U27)/(5*P27),0)</f>
@@ -2791,25 +2791,25 @@
         <v>0</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="P28" s="12" t="n">
-        <v>529</v>
+        <v>762</v>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>454</v>
+        <v>579</v>
       </c>
       <c r="R28" s="12" t="n">
-        <v>519</v>
+        <v>739</v>
       </c>
       <c r="S28" s="12" t="n">
-        <v>511</v>
+        <v>716</v>
       </c>
       <c r="T28" s="12" t="n">
-        <v>529</v>
+        <v>762</v>
       </c>
       <c r="U28" s="12" t="n">
-        <v>385</v>
+        <v>491</v>
       </c>
       <c r="V28" s="13">
         <f>IFERROR(SUM(Q28:U28)/(5*P28),0)</f>
@@ -2965,25 +2965,25 @@
         <v>0</v>
       </c>
       <c r="O30" s="12" t="n">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="P30" s="12" t="n">
-        <v>420</v>
+        <v>571</v>
       </c>
       <c r="Q30" s="12" t="n">
-        <v>254</v>
+        <v>338</v>
       </c>
       <c r="R30" s="12" t="n">
-        <v>300</v>
+        <v>412</v>
       </c>
       <c r="S30" s="12" t="n">
-        <v>351</v>
+        <v>483</v>
       </c>
       <c r="T30" s="12" t="n">
-        <v>420</v>
+        <v>571</v>
       </c>
       <c r="U30" s="12" t="n">
-        <v>272</v>
+        <v>365</v>
       </c>
       <c r="V30" s="13">
         <f>IFERROR(SUM(Q30:U30)/(5*P30),0)</f>
@@ -3052,25 +3052,25 @@
         <v>0</v>
       </c>
       <c r="O31" s="12" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="P31" s="12" t="n">
-        <v>226</v>
+        <v>259</v>
       </c>
       <c r="Q31" s="12" t="n">
-        <v>172</v>
+        <v>202</v>
       </c>
       <c r="R31" s="12" t="n">
-        <v>221</v>
+        <v>253</v>
       </c>
       <c r="S31" s="12" t="n">
-        <v>217</v>
+        <v>249</v>
       </c>
       <c r="T31" s="12" t="n">
-        <v>226</v>
+        <v>259</v>
       </c>
       <c r="U31" s="12" t="n">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="V31" s="13">
         <f>IFERROR(SUM(Q31:U31)/(5*P31),0)</f>
@@ -3226,25 +3226,25 @@
         <v>0</v>
       </c>
       <c r="O33" s="12" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="P33" s="12" t="n">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="Q33" s="12" t="n">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="R33" s="12" t="n">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="S33" s="12" t="n">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="T33" s="12" t="n">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="U33" s="12" t="n">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="V33" s="13">
         <f>IFERROR(SUM(Q33:U33)/(5*P33),0)</f>
@@ -3574,25 +3574,25 @@
         <v>0</v>
       </c>
       <c r="O37" s="12" t="n">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="P37" s="12" t="n">
-        <v>1200</v>
+        <v>1501</v>
       </c>
       <c r="Q37" s="12" t="n">
-        <v>781</v>
+        <v>941</v>
       </c>
       <c r="R37" s="12" t="n">
-        <v>1096</v>
+        <v>1377</v>
       </c>
       <c r="S37" s="12" t="n">
-        <v>1110</v>
+        <v>1395</v>
       </c>
       <c r="T37" s="12" t="n">
-        <v>1200</v>
+        <v>1501</v>
       </c>
       <c r="U37" s="12" t="n">
-        <v>912</v>
+        <v>1141</v>
       </c>
       <c r="V37" s="13">
         <f>IFERROR(SUM(Q37:U37)/(5*P37),0)</f>
@@ -3748,25 +3748,25 @@
         <v>0</v>
       </c>
       <c r="O39" s="12" t="n">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="P39" s="12" t="n">
-        <v>562</v>
+        <v>807</v>
       </c>
       <c r="Q39" s="12" t="n">
-        <v>465</v>
+        <v>643</v>
       </c>
       <c r="R39" s="12" t="n">
-        <v>506</v>
+        <v>718</v>
       </c>
       <c r="S39" s="12" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="T39" s="12" t="n">
-        <v>562</v>
+        <v>807</v>
       </c>
       <c r="U39" s="12" t="n">
-        <v>468</v>
+        <v>671</v>
       </c>
       <c r="V39" s="13">
         <f>IFERROR(SUM(Q39:U39)/(5*P39),0)</f>
@@ -4270,25 +4270,25 @@
         <v>0</v>
       </c>
       <c r="O45" s="12" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="P45" s="12" t="n">
-        <v>488</v>
+        <v>802</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>364</v>
+        <v>538</v>
       </c>
       <c r="R45" s="12" t="n">
-        <v>476</v>
+        <v>780</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>483</v>
+        <v>791</v>
       </c>
       <c r="T45" s="12" t="n">
-        <v>488</v>
+        <v>802</v>
       </c>
       <c r="U45" s="12" t="n">
-        <v>371</v>
+        <v>604</v>
       </c>
       <c r="V45" s="13">
         <f>IFERROR(SUM(Q45:U45)/(5*P45),0)</f>
@@ -4357,25 +4357,25 @@
         <v>0</v>
       </c>
       <c r="O46" s="12" t="n">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="P46" s="12" t="n">
-        <v>453</v>
+        <v>809</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>274</v>
+        <v>467</v>
       </c>
       <c r="R46" s="12" t="n">
-        <v>407</v>
+        <v>725</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>425</v>
+        <v>758</v>
       </c>
       <c r="T46" s="12" t="n">
-        <v>453</v>
+        <v>809</v>
       </c>
       <c r="U46" s="12" t="n">
-        <v>293</v>
+        <v>514</v>
       </c>
       <c r="V46" s="13">
         <f>IFERROR(SUM(Q46:U46)/(5*P46),0)</f>
@@ -4444,25 +4444,25 @@
         <v>0</v>
       </c>
       <c r="O47" s="12" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P47" s="12" t="n">
-        <v>234</v>
+        <v>264</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>201</v>
+        <v>229</v>
       </c>
       <c r="R47" s="12" t="n">
-        <v>231</v>
+        <v>261</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>231</v>
+        <v>261</v>
       </c>
       <c r="T47" s="12" t="n">
-        <v>234</v>
+        <v>264</v>
       </c>
       <c r="U47" s="12" t="n">
-        <v>210</v>
+        <v>235</v>
       </c>
       <c r="V47" s="13">
         <f>IFERROR(SUM(Q47:U47)/(5*P47),0)</f>
@@ -4531,25 +4531,25 @@
         <v>0</v>
       </c>
       <c r="O48" s="12" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="P48" s="12" t="n">
-        <v>231</v>
+        <v>276</v>
       </c>
       <c r="Q48" s="12" t="n">
-        <v>141</v>
+        <v>179</v>
       </c>
       <c r="R48" s="12" t="n">
-        <v>228</v>
+        <v>272</v>
       </c>
       <c r="S48" s="12" t="n">
-        <v>225</v>
+        <v>268</v>
       </c>
       <c r="T48" s="12" t="n">
-        <v>231</v>
+        <v>276</v>
       </c>
       <c r="U48" s="12" t="n">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="V48" s="13">
         <f>IFERROR(SUM(Q48:U48)/(5*P48),0)</f>
@@ -5140,25 +5140,25 @@
         <v>0</v>
       </c>
       <c r="O55" s="12" t="n">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="P55" s="12" t="n">
-        <v>529</v>
+        <v>848</v>
       </c>
       <c r="Q55" s="12" t="n">
-        <v>447</v>
+        <v>658</v>
       </c>
       <c r="R55" s="12" t="n">
-        <v>521</v>
+        <v>834</v>
       </c>
       <c r="S55" s="12" t="n">
-        <v>519</v>
+        <v>831</v>
       </c>
       <c r="T55" s="12" t="n">
-        <v>529</v>
+        <v>848</v>
       </c>
       <c r="U55" s="12" t="n">
-        <v>351</v>
+        <v>502</v>
       </c>
       <c r="V55" s="13">
         <f>IFERROR(SUM(Q55:U55)/(5*P55),0)</f>
@@ -5227,25 +5227,25 @@
         <v>0</v>
       </c>
       <c r="O56" s="12" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="P56" s="12" t="n">
-        <v>790</v>
+        <v>1249</v>
       </c>
       <c r="Q56" s="12" t="n">
-        <v>570</v>
+        <v>870</v>
       </c>
       <c r="R56" s="12" t="n">
-        <v>750</v>
+        <v>1191</v>
       </c>
       <c r="S56" s="12" t="n">
-        <v>776</v>
+        <v>1220</v>
       </c>
       <c r="T56" s="12" t="n">
-        <v>790</v>
+        <v>1249</v>
       </c>
       <c r="U56" s="12" t="n">
-        <v>526</v>
+        <v>820</v>
       </c>
       <c r="V56" s="13">
         <f>IFERROR(SUM(Q56:U56)/(5*P56),0)</f>
@@ -5314,25 +5314,25 @@
         <v>0</v>
       </c>
       <c r="O57" s="12" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="P57" s="12" t="n">
-        <v>240</v>
+        <v>291</v>
       </c>
       <c r="Q57" s="12" t="n">
-        <v>206</v>
+        <v>256</v>
       </c>
       <c r="R57" s="12" t="n">
-        <v>237</v>
+        <v>288</v>
       </c>
       <c r="S57" s="12" t="n">
-        <v>238</v>
+        <v>289</v>
       </c>
       <c r="T57" s="12" t="n">
-        <v>240</v>
+        <v>291</v>
       </c>
       <c r="U57" s="12" t="n">
-        <v>220</v>
+        <v>269</v>
       </c>
       <c r="V57" s="13">
         <f>IFERROR(SUM(Q57:U57)/(5*P57),0)</f>
@@ -5401,25 +5401,25 @@
         <v>0</v>
       </c>
       <c r="O58" s="12" t="n">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="P58" s="12" t="n">
-        <v>528</v>
+        <v>861</v>
       </c>
       <c r="Q58" s="12" t="n">
-        <v>375</v>
+        <v>549</v>
       </c>
       <c r="R58" s="12" t="n">
-        <v>516</v>
+        <v>838</v>
       </c>
       <c r="S58" s="12" t="n">
-        <v>522</v>
+        <v>847</v>
       </c>
       <c r="T58" s="12" t="n">
-        <v>528</v>
+        <v>861</v>
       </c>
       <c r="U58" s="12" t="n">
-        <v>401</v>
+        <v>583</v>
       </c>
       <c r="V58" s="13">
         <f>IFERROR(SUM(Q58:U58)/(5*P58),0)</f>
@@ -5488,25 +5488,25 @@
         <v>0</v>
       </c>
       <c r="O59" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="P59" s="12" t="n">
-        <v>184</v>
+        <v>219</v>
       </c>
       <c r="Q59" s="12" t="n">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="R59" s="12" t="n">
-        <v>179</v>
+        <v>212</v>
       </c>
       <c r="S59" s="12" t="n">
-        <v>182</v>
+        <v>216</v>
       </c>
       <c r="T59" s="12" t="n">
-        <v>184</v>
+        <v>219</v>
       </c>
       <c r="U59" s="12" t="n">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="V59" s="13">
         <f>IFERROR(SUM(Q59:U59)/(5*P59),0)</f>
@@ -5575,25 +5575,25 @@
         <v>0</v>
       </c>
       <c r="O60" s="12" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="P60" s="12" t="n">
-        <v>60</v>
+        <v>254</v>
       </c>
       <c r="Q60" s="12" t="n">
-        <v>52</v>
+        <v>202</v>
       </c>
       <c r="R60" s="12" t="n">
-        <v>58</v>
+        <v>248</v>
       </c>
       <c r="S60" s="12" t="n">
-        <v>60</v>
+        <v>250</v>
       </c>
       <c r="T60" s="12" t="n">
-        <v>60</v>
+        <v>254</v>
       </c>
       <c r="U60" s="12" t="n">
-        <v>43</v>
+        <v>169</v>
       </c>
       <c r="V60" s="13">
         <f>IFERROR(SUM(Q60:U60)/(5*P60),0)</f>
@@ -5662,25 +5662,25 @@
         <v>0</v>
       </c>
       <c r="O61" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P61" s="12" t="n">
-        <v>0</v>
+        <v>207</v>
       </c>
       <c r="Q61" s="12" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="R61" s="12" t="n">
-        <v>0</v>
+        <v>205</v>
       </c>
       <c r="S61" s="12" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="T61" s="12" t="n">
-        <v>0</v>
+        <v>207</v>
       </c>
       <c r="U61" s="12" t="n">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="V61" s="13">
         <f>IFERROR(SUM(Q61:U61)/(5*P61),0)</f>
@@ -5688,7 +5688,7 @@
       </c>
       <c r="W61" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X61" s="15" t="n"/>
@@ -5749,25 +5749,25 @@
         <v>0</v>
       </c>
       <c r="O62" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P62" s="12" t="n">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="Q62" s="12" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="R62" s="12" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="S62" s="12" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="T62" s="12" t="n">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="U62" s="12" t="n">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="V62" s="13">
         <f>IFERROR(SUM(Q62:U62)/(5*P62),0)</f>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="W62" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X62" s="15" t="n"/>
@@ -5836,25 +5836,25 @@
         <v>0</v>
       </c>
       <c r="O63" s="12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P63" s="12" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="Q63" s="12" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="R63" s="12" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="S63" s="12" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="T63" s="12" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="U63" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="V63" s="13">
         <f>IFERROR(SUM(Q63:U63)/(5*P63),0)</f>
@@ -5862,7 +5862,7 @@
       </c>
       <c r="W63" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X63" s="15" t="n"/>
@@ -5923,25 +5923,25 @@
         <v>0</v>
       </c>
       <c r="O64" s="12" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="P64" s="12" t="n">
-        <v>538</v>
+        <v>826</v>
       </c>
       <c r="Q64" s="12" t="n">
-        <v>404</v>
+        <v>577</v>
       </c>
       <c r="R64" s="12" t="n">
-        <v>524</v>
+        <v>801</v>
       </c>
       <c r="S64" s="12" t="n">
-        <v>531</v>
+        <v>807</v>
       </c>
       <c r="T64" s="12" t="n">
-        <v>538</v>
+        <v>826</v>
       </c>
       <c r="U64" s="12" t="n">
-        <v>372</v>
+        <v>532</v>
       </c>
       <c r="V64" s="13">
         <f>IFERROR(SUM(Q64:U64)/(5*P64),0)</f>
@@ -6010,25 +6010,25 @@
         <v>0</v>
       </c>
       <c r="O65" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P65" s="12" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="Q65" s="12" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="R65" s="12" t="n">
-        <v>0</v>
+        <v>231</v>
       </c>
       <c r="S65" s="12" t="n">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="T65" s="12" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="U65" s="12" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="V65" s="13">
         <f>IFERROR(SUM(Q65:U65)/(5*P65),0)</f>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="W65" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Discovering</t>
         </is>
       </c>
       <c r="X65" s="15" t="n"/>
@@ -6097,25 +6097,25 @@
         <v>0</v>
       </c>
       <c r="O66" s="12" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="P66" s="12" t="n">
-        <v>538</v>
+        <v>882</v>
       </c>
       <c r="Q66" s="12" t="n">
-        <v>282</v>
+        <v>395</v>
       </c>
       <c r="R66" s="12" t="n">
-        <v>526</v>
+        <v>859</v>
       </c>
       <c r="S66" s="12" t="n">
-        <v>531</v>
+        <v>858</v>
       </c>
       <c r="T66" s="12" t="n">
-        <v>538</v>
+        <v>882</v>
       </c>
       <c r="U66" s="12" t="n">
-        <v>318</v>
+        <v>437</v>
       </c>
       <c r="V66" s="13">
         <f>IFERROR(SUM(Q66:U66)/(5*P66),0)</f>
@@ -6271,25 +6271,25 @@
         <v>0</v>
       </c>
       <c r="O68" s="12" t="n">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="P68" s="12" t="n">
-        <v>364</v>
+        <v>558</v>
       </c>
       <c r="Q68" s="12" t="n">
-        <v>265</v>
+        <v>362</v>
       </c>
       <c r="R68" s="12" t="n">
-        <v>353</v>
+        <v>539</v>
       </c>
       <c r="S68" s="12" t="n">
-        <v>357</v>
+        <v>535</v>
       </c>
       <c r="T68" s="12" t="n">
-        <v>364</v>
+        <v>558</v>
       </c>
       <c r="U68" s="12" t="n">
-        <v>266</v>
+        <v>365</v>
       </c>
       <c r="V68" s="13">
         <f>IFERROR(SUM(Q68:U68)/(5*P68),0)</f>
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>2986</v>
+        <v>2061</v>
       </c>
     </row>
   </sheetData>
@@ -6972,7 +6972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7006,7 +7006,7 @@
     <row r="2">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>full-uae</t>
+          <t>chains</t>
         </is>
       </c>
       <c r="B2" s="21" t="inlineStr">
@@ -7015,47 +7015,101 @@
         </is>
       </c>
       <c r="C2" s="21" t="n">
-        <v>1917</v>
+        <v>210</v>
       </c>
       <c r="D2" s="21" t="n">
-        <v>21244</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
+          <t>full-uae</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="n">
+        <v>1989</v>
+      </c>
+      <c r="D3" s="21" t="n">
+        <v>22182</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>more-areas</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>432</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>6162</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>northern-emirates</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>210</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>3467</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
           <t>pilot-dubai</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C6" s="21" t="n">
         <v>97</v>
       </c>
-      <c r="D3" s="21" t="n">
+      <c r="D6" s="21" t="n">
         <v>1621</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C4" s="25">
-        <f>SUM(C2:C3)</f>
-        <v/>
-      </c>
-      <c r="D4" s="25">
-        <f>SUM(D2:D3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="C7" s="25">
+        <f>SUM(C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="25">
+        <f>SUM(D2:D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Unique places per run; the Tracker deduplicates across runs, so its total can be lower.</t>
         </is>

</xml_diff>

<commit_message>
Discovery batch 4: Northern Emirates sparse categories, Abu Dhabi/Al Ain areas, chains 71-180
- serp-discovery.ts: runs northern-sparse, abu-dhabi-areas and chains-2
  (next 110 chains ranked across all runs, skipping ones already searched).
- Tracker: 3,820 searches total, 36,469 unique businesses.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reviewencer-data-tracker.xlsx
+++ b/docs/Reviewencer-data-tracker.xlsx
@@ -331,7 +331,7 @@
     </comment>
     <comment ref="B18" authorId="0" shapeId="0">
       <text>
-        <t>Read from the SerpAPI account page at 2026-10-21 19:43 (free lookup). Refreshes when the tracker is regenerated.</t>
+        <t>Read from the SerpAPI account page at 2026-10-21 23:01 (free lookup). Refreshes when the tracker is regenerated.</t>
       </text>
     </comment>
   </commentList>
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-21 19:43 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
+          <t>Generated 2026-10-21 23:01 from the live database (11,039 businesses) and SerpAPI discovery runs in data/serp/. Refresh: python scripts/data_tracker.py</t>
         </is>
       </c>
     </row>
@@ -877,25 +877,25 @@
         <v>0</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>176</v>
+        <v>209</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>2487</v>
+        <v>2770</v>
       </c>
       <c r="Q6" s="12" t="n">
-        <v>1781</v>
+        <v>1968</v>
       </c>
       <c r="R6" s="12" t="n">
-        <v>2432</v>
+        <v>2704</v>
       </c>
       <c r="S6" s="12" t="n">
-        <v>2452</v>
+        <v>2727</v>
       </c>
       <c r="T6" s="12" t="n">
-        <v>2487</v>
+        <v>2770</v>
       </c>
       <c r="U6" s="12" t="n">
-        <v>2420</v>
+        <v>2679</v>
       </c>
       <c r="V6" s="13">
         <f>IFERROR(SUM(Q6:U6)/(5*P6),0)</f>
@@ -964,25 +964,25 @@
         <v>0</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>144</v>
+        <v>183</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>2349</v>
+        <v>2647</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>1669</v>
+        <v>1870</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>2222</v>
+        <v>2493</v>
       </c>
       <c r="S7" s="12" t="n">
-        <v>2296</v>
+        <v>2573</v>
       </c>
       <c r="T7" s="12" t="n">
-        <v>2349</v>
+        <v>2647</v>
       </c>
       <c r="U7" s="12" t="n">
-        <v>2140</v>
+        <v>2377</v>
       </c>
       <c r="V7" s="13">
         <f>IFERROR(SUM(Q7:U7)/(5*P7),0)</f>
@@ -1051,25 +1051,25 @@
         <v>0</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>1358</v>
+        <v>1586</v>
       </c>
       <c r="Q8" s="12" t="n">
-        <v>968</v>
+        <v>1109</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>1330</v>
+        <v>1556</v>
       </c>
       <c r="S8" s="12" t="n">
-        <v>1344</v>
+        <v>1568</v>
       </c>
       <c r="T8" s="12" t="n">
-        <v>1358</v>
+        <v>1586</v>
       </c>
       <c r="U8" s="12" t="n">
-        <v>1321</v>
+        <v>1531</v>
       </c>
       <c r="V8" s="13">
         <f>IFERROR(SUM(Q8:U8)/(5*P8),0)</f>
@@ -1138,25 +1138,25 @@
         <v>0</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>1099</v>
+        <v>1333</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>730</v>
+        <v>886</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>1056</v>
+        <v>1255</v>
       </c>
       <c r="S9" s="12" t="n">
-        <v>1076</v>
+        <v>1302</v>
       </c>
       <c r="T9" s="12" t="n">
-        <v>1099</v>
+        <v>1333</v>
       </c>
       <c r="U9" s="12" t="n">
-        <v>942</v>
+        <v>1123</v>
       </c>
       <c r="V9" s="13">
         <f>IFERROR(SUM(Q9:U9)/(5*P9),0)</f>
@@ -1225,25 +1225,25 @@
         <v>0</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="P10" s="12" t="n">
-        <v>1195</v>
+        <v>1371</v>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>855</v>
+        <v>973</v>
       </c>
       <c r="R10" s="12" t="n">
-        <v>1148</v>
+        <v>1320</v>
       </c>
       <c r="S10" s="12" t="n">
-        <v>1179</v>
+        <v>1352</v>
       </c>
       <c r="T10" s="12" t="n">
-        <v>1195</v>
+        <v>1371</v>
       </c>
       <c r="U10" s="12" t="n">
-        <v>1072</v>
+        <v>1220</v>
       </c>
       <c r="V10" s="13">
         <f>IFERROR(SUM(Q10:U10)/(5*P10),0)</f>
@@ -1312,25 +1312,25 @@
         <v>0</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="P11" s="12" t="n">
-        <v>197</v>
+        <v>326</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>158</v>
+        <v>239</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>187</v>
+        <v>300</v>
       </c>
       <c r="S11" s="12" t="n">
-        <v>189</v>
+        <v>302</v>
       </c>
       <c r="T11" s="12" t="n">
-        <v>197</v>
+        <v>326</v>
       </c>
       <c r="U11" s="12" t="n">
-        <v>177</v>
+        <v>268</v>
       </c>
       <c r="V11" s="13">
         <f>IFERROR(SUM(Q11:U11)/(5*P11),0)</f>
@@ -1399,25 +1399,25 @@
         <v>0</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="P12" s="12" t="n">
-        <v>152</v>
+        <v>244</v>
       </c>
       <c r="Q12" s="12" t="n">
-        <v>88</v>
+        <v>132</v>
       </c>
       <c r="R12" s="12" t="n">
-        <v>128</v>
+        <v>209</v>
       </c>
       <c r="S12" s="12" t="n">
-        <v>139</v>
+        <v>222</v>
       </c>
       <c r="T12" s="12" t="n">
-        <v>152</v>
+        <v>244</v>
       </c>
       <c r="U12" s="12" t="n">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="V12" s="13">
         <f>IFERROR(SUM(Q12:U12)/(5*P12),0)</f>
@@ -1486,25 +1486,25 @@
         <v>0</v>
       </c>
       <c r="O13" s="12" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="P13" s="12" t="n">
-        <v>164</v>
+        <v>323</v>
       </c>
       <c r="Q13" s="12" t="n">
-        <v>111</v>
+        <v>167</v>
       </c>
       <c r="R13" s="12" t="n">
-        <v>161</v>
+        <v>315</v>
       </c>
       <c r="S13" s="12" t="n">
-        <v>161</v>
+        <v>314</v>
       </c>
       <c r="T13" s="12" t="n">
-        <v>164</v>
+        <v>323</v>
       </c>
       <c r="U13" s="12" t="n">
-        <v>130</v>
+        <v>226</v>
       </c>
       <c r="V13" s="13">
         <f>IFERROR(SUM(Q13:U13)/(5*P13),0)</f>
@@ -1573,25 +1573,25 @@
         <v>0</v>
       </c>
       <c r="O14" s="12" t="n">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="P14" s="12" t="n">
-        <v>1419</v>
+        <v>1665</v>
       </c>
       <c r="Q14" s="12" t="n">
-        <v>896</v>
+        <v>1022</v>
       </c>
       <c r="R14" s="12" t="n">
-        <v>1348</v>
+        <v>1571</v>
       </c>
       <c r="S14" s="12" t="n">
-        <v>1388</v>
+        <v>1624</v>
       </c>
       <c r="T14" s="12" t="n">
-        <v>1419</v>
+        <v>1665</v>
       </c>
       <c r="U14" s="12" t="n">
-        <v>1218</v>
+        <v>1399</v>
       </c>
       <c r="V14" s="13">
         <f>IFERROR(SUM(Q14:U14)/(5*P14),0)</f>
@@ -1660,25 +1660,25 @@
         <v>0</v>
       </c>
       <c r="O15" s="12" t="n">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="P15" s="12" t="n">
-        <v>742</v>
+        <v>828</v>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>402</v>
+        <v>438</v>
       </c>
       <c r="R15" s="12" t="n">
-        <v>669</v>
+        <v>749</v>
       </c>
       <c r="S15" s="12" t="n">
-        <v>717</v>
+        <v>794</v>
       </c>
       <c r="T15" s="12" t="n">
-        <v>742</v>
+        <v>828</v>
       </c>
       <c r="U15" s="12" t="n">
-        <v>543</v>
+        <v>600</v>
       </c>
       <c r="V15" s="13">
         <f>IFERROR(SUM(Q15:U15)/(5*P15),0)</f>
@@ -1747,25 +1747,25 @@
         <v>0</v>
       </c>
       <c r="O16" s="12" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="P16" s="12" t="n">
-        <v>126</v>
+        <v>199</v>
       </c>
       <c r="Q16" s="12" t="n">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="R16" s="12" t="n">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="S16" s="12" t="n">
-        <v>112</v>
+        <v>178</v>
       </c>
       <c r="T16" s="12" t="n">
-        <v>126</v>
+        <v>199</v>
       </c>
       <c r="U16" s="12" t="n">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="V16" s="13">
         <f>IFERROR(SUM(Q16:U16)/(5*P16),0)</f>
@@ -1834,25 +1834,25 @@
         <v>0</v>
       </c>
       <c r="O17" s="12" t="n">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="P17" s="12" t="n">
-        <v>1754</v>
+        <v>1927</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>1432</v>
+        <v>1567</v>
       </c>
       <c r="R17" s="12" t="n">
-        <v>1693</v>
+        <v>1853</v>
       </c>
       <c r="S17" s="12" t="n">
-        <v>1681</v>
+        <v>1841</v>
       </c>
       <c r="T17" s="12" t="n">
-        <v>1754</v>
+        <v>1927</v>
       </c>
       <c r="U17" s="12" t="n">
-        <v>1443</v>
+        <v>1575</v>
       </c>
       <c r="V17" s="13">
         <f>IFERROR(SUM(Q17:U17)/(5*P17),0)</f>
@@ -1921,25 +1921,25 @@
         <v>0</v>
       </c>
       <c r="O18" s="12" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="P18" s="12" t="n">
-        <v>134</v>
+        <v>223</v>
       </c>
       <c r="Q18" s="12" t="n">
-        <v>126</v>
+        <v>189</v>
       </c>
       <c r="R18" s="12" t="n">
-        <v>126</v>
+        <v>213</v>
       </c>
       <c r="S18" s="12" t="n">
-        <v>129</v>
+        <v>217</v>
       </c>
       <c r="T18" s="12" t="n">
-        <v>134</v>
+        <v>223</v>
       </c>
       <c r="U18" s="12" t="n">
-        <v>122</v>
+        <v>195</v>
       </c>
       <c r="V18" s="13">
         <f>IFERROR(SUM(Q18:U18)/(5*P18),0)</f>
@@ -2008,25 +2008,25 @@
         <v>0</v>
       </c>
       <c r="O19" s="12" t="n">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="P19" s="12" t="n">
-        <v>1131</v>
+        <v>1267</v>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>971</v>
+        <v>1081</v>
       </c>
       <c r="R19" s="12" t="n">
-        <v>1118</v>
+        <v>1252</v>
       </c>
       <c r="S19" s="12" t="n">
-        <v>1108</v>
+        <v>1243</v>
       </c>
       <c r="T19" s="12" t="n">
-        <v>1131</v>
+        <v>1267</v>
       </c>
       <c r="U19" s="12" t="n">
-        <v>1008</v>
+        <v>1128</v>
       </c>
       <c r="V19" s="13">
         <f>IFERROR(SUM(Q19:U19)/(5*P19),0)</f>
@@ -2095,25 +2095,25 @@
         <v>0</v>
       </c>
       <c r="O20" s="12" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="P20" s="12" t="n">
-        <v>899</v>
+        <v>988</v>
       </c>
       <c r="Q20" s="12" t="n">
-        <v>746</v>
+        <v>816</v>
       </c>
       <c r="R20" s="12" t="n">
-        <v>881</v>
+        <v>966</v>
       </c>
       <c r="S20" s="12" t="n">
-        <v>880</v>
+        <v>967</v>
       </c>
       <c r="T20" s="12" t="n">
-        <v>899</v>
+        <v>988</v>
       </c>
       <c r="U20" s="12" t="n">
-        <v>780</v>
+        <v>854</v>
       </c>
       <c r="V20" s="13">
         <f>IFERROR(SUM(Q20:U20)/(5*P20),0)</f>
@@ -2182,25 +2182,25 @@
         <v>0</v>
       </c>
       <c r="O21" s="12" t="n">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="P21" s="12" t="n">
-        <v>1377</v>
+        <v>1479</v>
       </c>
       <c r="Q21" s="12" t="n">
-        <v>1119</v>
+        <v>1197</v>
       </c>
       <c r="R21" s="12" t="n">
-        <v>1359</v>
+        <v>1456</v>
       </c>
       <c r="S21" s="12" t="n">
-        <v>1353</v>
+        <v>1451</v>
       </c>
       <c r="T21" s="12" t="n">
-        <v>1377</v>
+        <v>1479</v>
       </c>
       <c r="U21" s="12" t="n">
-        <v>1166</v>
+        <v>1249</v>
       </c>
       <c r="V21" s="13">
         <f>IFERROR(SUM(Q21:U21)/(5*P21),0)</f>
@@ -2269,25 +2269,25 @@
         <v>0</v>
       </c>
       <c r="O22" s="12" t="n">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="P22" s="12" t="n">
-        <v>1344</v>
+        <v>1589</v>
       </c>
       <c r="Q22" s="12" t="n">
-        <v>1081</v>
+        <v>1261</v>
       </c>
       <c r="R22" s="12" t="n">
-        <v>1325</v>
+        <v>1563</v>
       </c>
       <c r="S22" s="12" t="n">
-        <v>1324</v>
+        <v>1560</v>
       </c>
       <c r="T22" s="12" t="n">
-        <v>1344</v>
+        <v>1589</v>
       </c>
       <c r="U22" s="12" t="n">
-        <v>1026</v>
+        <v>1177</v>
       </c>
       <c r="V22" s="13">
         <f>IFERROR(SUM(Q22:U22)/(5*P22),0)</f>
@@ -2356,25 +2356,25 @@
         <v>0</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="P23" s="12" t="n">
-        <v>854</v>
+        <v>966</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>586</v>
+        <v>656</v>
       </c>
       <c r="R23" s="12" t="n">
-        <v>841</v>
+        <v>950</v>
       </c>
       <c r="S23" s="12" t="n">
-        <v>833</v>
+        <v>942</v>
       </c>
       <c r="T23" s="12" t="n">
-        <v>854</v>
+        <v>966</v>
       </c>
       <c r="U23" s="12" t="n">
-        <v>600</v>
+        <v>656</v>
       </c>
       <c r="V23" s="13">
         <f>IFERROR(SUM(Q23:U23)/(5*P23),0)</f>
@@ -2443,25 +2443,25 @@
         <v>0</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="P24" s="12" t="n">
-        <v>1878</v>
+        <v>2060</v>
       </c>
       <c r="Q24" s="12" t="n">
-        <v>1351</v>
+        <v>1481</v>
       </c>
       <c r="R24" s="12" t="n">
-        <v>1806</v>
+        <v>1988</v>
       </c>
       <c r="S24" s="12" t="n">
-        <v>1853</v>
+        <v>2033</v>
       </c>
       <c r="T24" s="12" t="n">
-        <v>1878</v>
+        <v>2060</v>
       </c>
       <c r="U24" s="12" t="n">
-        <v>1630</v>
+        <v>1785</v>
       </c>
       <c r="V24" s="13">
         <f>IFERROR(SUM(Q24:U24)/(5*P24),0)</f>
@@ -2530,25 +2530,25 @@
         <v>0</v>
       </c>
       <c r="O25" s="12" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="P25" s="12" t="n">
-        <v>173</v>
+        <v>325</v>
       </c>
       <c r="Q25" s="12" t="n">
-        <v>154</v>
+        <v>259</v>
       </c>
       <c r="R25" s="12" t="n">
-        <v>170</v>
+        <v>319</v>
       </c>
       <c r="S25" s="12" t="n">
-        <v>169</v>
+        <v>320</v>
       </c>
       <c r="T25" s="12" t="n">
-        <v>173</v>
+        <v>325</v>
       </c>
       <c r="U25" s="12" t="n">
-        <v>147</v>
+        <v>259</v>
       </c>
       <c r="V25" s="13">
         <f>IFERROR(SUM(Q25:U25)/(5*P25),0)</f>
@@ -2617,25 +2617,25 @@
         <v>0</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="P26" s="12" t="n">
-        <v>203</v>
+        <v>251</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="R26" s="12" t="n">
-        <v>193</v>
+        <v>240</v>
       </c>
       <c r="S26" s="12" t="n">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="T26" s="12" t="n">
-        <v>203</v>
+        <v>251</v>
       </c>
       <c r="U26" s="12" t="n">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="V26" s="13">
         <f>IFERROR(SUM(Q26:U26)/(5*P26),0)</f>
@@ -2704,25 +2704,25 @@
         <v>0</v>
       </c>
       <c r="O27" s="12" t="n">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="P27" s="12" t="n">
-        <v>527</v>
+        <v>576</v>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>470</v>
+        <v>506</v>
       </c>
       <c r="R27" s="12" t="n">
-        <v>510</v>
+        <v>558</v>
       </c>
       <c r="S27" s="12" t="n">
-        <v>492</v>
+        <v>537</v>
       </c>
       <c r="T27" s="12" t="n">
-        <v>527</v>
+        <v>576</v>
       </c>
       <c r="U27" s="12" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="V27" s="13">
         <f>IFERROR(SUM(Q27:U27)/(5*P27),0)</f>
@@ -2791,25 +2791,25 @@
         <v>0</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="P28" s="12" t="n">
-        <v>762</v>
+        <v>860</v>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>579</v>
+        <v>637</v>
       </c>
       <c r="R28" s="12" t="n">
-        <v>739</v>
+        <v>833</v>
       </c>
       <c r="S28" s="12" t="n">
-        <v>716</v>
+        <v>801</v>
       </c>
       <c r="T28" s="12" t="n">
-        <v>762</v>
+        <v>860</v>
       </c>
       <c r="U28" s="12" t="n">
-        <v>491</v>
+        <v>548</v>
       </c>
       <c r="V28" s="13">
         <f>IFERROR(SUM(Q28:U28)/(5*P28),0)</f>
@@ -2878,25 +2878,25 @@
         <v>0</v>
       </c>
       <c r="O29" s="12" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="P29" s="12" t="n">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="Q29" s="12" t="n">
-        <v>88</v>
+        <v>131</v>
       </c>
       <c r="R29" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="S29" s="12" t="n">
+        <v>157</v>
+      </c>
+      <c r="T29" s="12" t="n">
+        <v>171</v>
+      </c>
+      <c r="U29" s="12" t="n">
         <v>97</v>
-      </c>
-      <c r="S29" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="T29" s="12" t="n">
-        <v>99</v>
-      </c>
-      <c r="U29" s="12" t="n">
-        <v>70</v>
       </c>
       <c r="V29" s="13">
         <f>IFERROR(SUM(Q29:U29)/(5*P29),0)</f>
@@ -2965,25 +2965,25 @@
         <v>0</v>
       </c>
       <c r="O30" s="12" t="n">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="P30" s="12" t="n">
-        <v>571</v>
+        <v>663</v>
       </c>
       <c r="Q30" s="12" t="n">
-        <v>338</v>
+        <v>385</v>
       </c>
       <c r="R30" s="12" t="n">
-        <v>412</v>
+        <v>471</v>
       </c>
       <c r="S30" s="12" t="n">
-        <v>483</v>
+        <v>552</v>
       </c>
       <c r="T30" s="12" t="n">
-        <v>571</v>
+        <v>663</v>
       </c>
       <c r="U30" s="12" t="n">
-        <v>365</v>
+        <v>427</v>
       </c>
       <c r="V30" s="13">
         <f>IFERROR(SUM(Q30:U30)/(5*P30),0)</f>
@@ -3052,25 +3052,25 @@
         <v>0</v>
       </c>
       <c r="O31" s="12" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="P31" s="12" t="n">
-        <v>259</v>
+        <v>443</v>
       </c>
       <c r="Q31" s="12" t="n">
-        <v>202</v>
+        <v>317</v>
       </c>
       <c r="R31" s="12" t="n">
-        <v>253</v>
+        <v>433</v>
       </c>
       <c r="S31" s="12" t="n">
-        <v>249</v>
+        <v>425</v>
       </c>
       <c r="T31" s="12" t="n">
-        <v>259</v>
+        <v>443</v>
       </c>
       <c r="U31" s="12" t="n">
-        <v>164</v>
+        <v>262</v>
       </c>
       <c r="V31" s="13">
         <f>IFERROR(SUM(Q31:U31)/(5*P31),0)</f>
@@ -3139,25 +3139,25 @@
         <v>0</v>
       </c>
       <c r="O32" s="12" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="P32" s="12" t="n">
-        <v>177</v>
+        <v>308</v>
       </c>
       <c r="Q32" s="12" t="n">
-        <v>140</v>
+        <v>222</v>
       </c>
       <c r="R32" s="12" t="n">
-        <v>175</v>
+        <v>295</v>
       </c>
       <c r="S32" s="12" t="n">
-        <v>167</v>
+        <v>269</v>
       </c>
       <c r="T32" s="12" t="n">
-        <v>177</v>
+        <v>308</v>
       </c>
       <c r="U32" s="12" t="n">
-        <v>135</v>
+        <v>233</v>
       </c>
       <c r="V32" s="13">
         <f>IFERROR(SUM(Q32:U32)/(5*P32),0)</f>
@@ -3226,25 +3226,25 @@
         <v>0</v>
       </c>
       <c r="O33" s="12" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="P33" s="12" t="n">
-        <v>216</v>
+        <v>284</v>
       </c>
       <c r="Q33" s="12" t="n">
-        <v>188</v>
+        <v>229</v>
       </c>
       <c r="R33" s="12" t="n">
-        <v>209</v>
+        <v>273</v>
       </c>
       <c r="S33" s="12" t="n">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="T33" s="12" t="n">
-        <v>216</v>
+        <v>284</v>
       </c>
       <c r="U33" s="12" t="n">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="V33" s="13">
         <f>IFERROR(SUM(Q33:U33)/(5*P33),0)</f>
@@ -3313,25 +3313,25 @@
         <v>0</v>
       </c>
       <c r="O34" s="12" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="P34" s="12" t="n">
-        <v>156</v>
+        <v>284</v>
       </c>
       <c r="Q34" s="12" t="n">
-        <v>120</v>
+        <v>204</v>
       </c>
       <c r="R34" s="12" t="n">
-        <v>130</v>
+        <v>227</v>
       </c>
       <c r="S34" s="12" t="n">
-        <v>115</v>
+        <v>166</v>
       </c>
       <c r="T34" s="12" t="n">
-        <v>156</v>
+        <v>284</v>
       </c>
       <c r="U34" s="12" t="n">
-        <v>144</v>
+        <v>255</v>
       </c>
       <c r="V34" s="13">
         <f>IFERROR(SUM(Q34:U34)/(5*P34),0)</f>
@@ -3400,25 +3400,25 @@
         <v>0</v>
       </c>
       <c r="O35" s="12" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="P35" s="12" t="n">
+        <v>94</v>
+      </c>
+      <c r="Q35" s="12" t="n">
         <v>79</v>
       </c>
-      <c r="Q35" s="12" t="n">
-        <v>67</v>
-      </c>
       <c r="R35" s="12" t="n">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="S35" s="12" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="T35" s="12" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="U35" s="12" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="V35" s="13">
         <f>IFERROR(SUM(Q35:U35)/(5*P35),0)</f>
@@ -3487,25 +3487,25 @@
         <v>0</v>
       </c>
       <c r="O36" s="12" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="P36" s="12" t="n">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="Q36" s="12" t="n">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="R36" s="12" t="n">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="S36" s="12" t="n">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="T36" s="12" t="n">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="U36" s="12" t="n">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="V36" s="13">
         <f>IFERROR(SUM(Q36:U36)/(5*P36),0)</f>
@@ -3574,25 +3574,25 @@
         <v>0</v>
       </c>
       <c r="O37" s="12" t="n">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="P37" s="12" t="n">
-        <v>1501</v>
+        <v>1582</v>
       </c>
       <c r="Q37" s="12" t="n">
-        <v>941</v>
+        <v>975</v>
       </c>
       <c r="R37" s="12" t="n">
-        <v>1377</v>
+        <v>1441</v>
       </c>
       <c r="S37" s="12" t="n">
-        <v>1395</v>
+        <v>1469</v>
       </c>
       <c r="T37" s="12" t="n">
-        <v>1501</v>
+        <v>1582</v>
       </c>
       <c r="U37" s="12" t="n">
-        <v>1141</v>
+        <v>1187</v>
       </c>
       <c r="V37" s="13">
         <f>IFERROR(SUM(Q37:U37)/(5*P37),0)</f>
@@ -3661,25 +3661,25 @@
         <v>0</v>
       </c>
       <c r="O38" s="12" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="P38" s="12" t="n">
-        <v>187</v>
+        <v>331</v>
       </c>
       <c r="Q38" s="12" t="n">
-        <v>145</v>
+        <v>210</v>
       </c>
       <c r="R38" s="12" t="n">
-        <v>152</v>
+        <v>242</v>
       </c>
       <c r="S38" s="12" t="n">
-        <v>174</v>
+        <v>279</v>
       </c>
       <c r="T38" s="12" t="n">
-        <v>187</v>
+        <v>331</v>
       </c>
       <c r="U38" s="12" t="n">
-        <v>173</v>
+        <v>287</v>
       </c>
       <c r="V38" s="13">
         <f>IFERROR(SUM(Q38:U38)/(5*P38),0)</f>
@@ -3748,25 +3748,25 @@
         <v>0</v>
       </c>
       <c r="O39" s="12" t="n">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="P39" s="12" t="n">
-        <v>807</v>
+        <v>853</v>
       </c>
       <c r="Q39" s="12" t="n">
-        <v>643</v>
+        <v>670</v>
       </c>
       <c r="R39" s="12" t="n">
-        <v>718</v>
+        <v>749</v>
       </c>
       <c r="S39" s="12" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="T39" s="12" t="n">
-        <v>807</v>
+        <v>853</v>
       </c>
       <c r="U39" s="12" t="n">
-        <v>671</v>
+        <v>690</v>
       </c>
       <c r="V39" s="13">
         <f>IFERROR(SUM(Q39:U39)/(5*P39),0)</f>
@@ -3835,25 +3835,25 @@
         <v>0</v>
       </c>
       <c r="O40" s="12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P40" s="12" t="n">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="Q40" s="12" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="R40" s="12" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="S40" s="12" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="T40" s="12" t="n">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="U40" s="12" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="V40" s="13">
         <f>IFERROR(SUM(Q40:U40)/(5*P40),0)</f>
@@ -3922,25 +3922,25 @@
         <v>0</v>
       </c>
       <c r="O41" s="12" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="P41" s="12" t="n">
-        <v>197</v>
+        <v>324</v>
       </c>
       <c r="Q41" s="12" t="n">
-        <v>130</v>
+        <v>189</v>
       </c>
       <c r="R41" s="12" t="n">
-        <v>181</v>
+        <v>273</v>
       </c>
       <c r="S41" s="12" t="n">
-        <v>182</v>
+        <v>276</v>
       </c>
       <c r="T41" s="12" t="n">
-        <v>197</v>
+        <v>324</v>
       </c>
       <c r="U41" s="12" t="n">
-        <v>154</v>
+        <v>218</v>
       </c>
       <c r="V41" s="13">
         <f>IFERROR(SUM(Q41:U41)/(5*P41),0)</f>
@@ -4009,25 +4009,25 @@
         <v>0</v>
       </c>
       <c r="O42" s="12" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="P42" s="12" t="n">
-        <v>230</v>
+        <v>370</v>
       </c>
       <c r="Q42" s="12" t="n">
-        <v>214</v>
+        <v>310</v>
       </c>
       <c r="R42" s="12" t="n">
-        <v>221</v>
+        <v>357</v>
       </c>
       <c r="S42" s="12" t="n">
-        <v>224</v>
+        <v>352</v>
       </c>
       <c r="T42" s="12" t="n">
-        <v>230</v>
+        <v>370</v>
       </c>
       <c r="U42" s="12" t="n">
-        <v>211</v>
+        <v>303</v>
       </c>
       <c r="V42" s="13">
         <f>IFERROR(SUM(Q42:U42)/(5*P42),0)</f>
@@ -4183,25 +4183,25 @@
         <v>0</v>
       </c>
       <c r="O44" s="12" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P44" s="12" t="n">
-        <v>238</v>
+        <v>393</v>
       </c>
       <c r="Q44" s="12" t="n">
-        <v>206</v>
+        <v>312</v>
       </c>
       <c r="R44" s="12" t="n">
-        <v>233</v>
+        <v>386</v>
       </c>
       <c r="S44" s="12" t="n">
-        <v>234</v>
+        <v>387</v>
       </c>
       <c r="T44" s="12" t="n">
-        <v>238</v>
+        <v>393</v>
       </c>
       <c r="U44" s="12" t="n">
-        <v>197</v>
+        <v>292</v>
       </c>
       <c r="V44" s="13">
         <f>IFERROR(SUM(Q44:U44)/(5*P44),0)</f>
@@ -4270,25 +4270,25 @@
         <v>0</v>
       </c>
       <c r="O45" s="12" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="P45" s="12" t="n">
-        <v>802</v>
+        <v>890</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>538</v>
+        <v>575</v>
       </c>
       <c r="R45" s="12" t="n">
-        <v>780</v>
+        <v>863</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>791</v>
+        <v>868</v>
       </c>
       <c r="T45" s="12" t="n">
-        <v>802</v>
+        <v>890</v>
       </c>
       <c r="U45" s="12" t="n">
-        <v>604</v>
+        <v>652</v>
       </c>
       <c r="V45" s="13">
         <f>IFERROR(SUM(Q45:U45)/(5*P45),0)</f>
@@ -4357,25 +4357,25 @@
         <v>0</v>
       </c>
       <c r="O46" s="12" t="n">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="P46" s="12" t="n">
-        <v>809</v>
+        <v>980</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>467</v>
+        <v>553</v>
       </c>
       <c r="R46" s="12" t="n">
-        <v>725</v>
+        <v>877</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>758</v>
+        <v>914</v>
       </c>
       <c r="T46" s="12" t="n">
-        <v>809</v>
+        <v>980</v>
       </c>
       <c r="U46" s="12" t="n">
-        <v>514</v>
+        <v>599</v>
       </c>
       <c r="V46" s="13">
         <f>IFERROR(SUM(Q46:U46)/(5*P46),0)</f>
@@ -4444,25 +4444,25 @@
         <v>0</v>
       </c>
       <c r="O47" s="12" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="P47" s="12" t="n">
-        <v>264</v>
+        <v>439</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>229</v>
+        <v>319</v>
       </c>
       <c r="R47" s="12" t="n">
-        <v>261</v>
+        <v>431</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>261</v>
+        <v>418</v>
       </c>
       <c r="T47" s="12" t="n">
-        <v>264</v>
+        <v>439</v>
       </c>
       <c r="U47" s="12" t="n">
-        <v>235</v>
+        <v>337</v>
       </c>
       <c r="V47" s="13">
         <f>IFERROR(SUM(Q47:U47)/(5*P47),0)</f>
@@ -4531,25 +4531,25 @@
         <v>0</v>
       </c>
       <c r="O48" s="12" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P48" s="12" t="n">
-        <v>276</v>
+        <v>415</v>
       </c>
       <c r="Q48" s="12" t="n">
-        <v>179</v>
+        <v>261</v>
       </c>
       <c r="R48" s="12" t="n">
-        <v>272</v>
+        <v>409</v>
       </c>
       <c r="S48" s="12" t="n">
-        <v>268</v>
+        <v>399</v>
       </c>
       <c r="T48" s="12" t="n">
-        <v>276</v>
+        <v>415</v>
       </c>
       <c r="U48" s="12" t="n">
-        <v>226</v>
+        <v>321</v>
       </c>
       <c r="V48" s="13">
         <f>IFERROR(SUM(Q48:U48)/(5*P48),0)</f>
@@ -5140,25 +5140,25 @@
         <v>0</v>
       </c>
       <c r="O55" s="12" t="n">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="P55" s="12" t="n">
-        <v>848</v>
+        <v>946</v>
       </c>
       <c r="Q55" s="12" t="n">
-        <v>658</v>
+        <v>714</v>
       </c>
       <c r="R55" s="12" t="n">
-        <v>834</v>
+        <v>926</v>
       </c>
       <c r="S55" s="12" t="n">
-        <v>831</v>
+        <v>925</v>
       </c>
       <c r="T55" s="12" t="n">
-        <v>848</v>
+        <v>946</v>
       </c>
       <c r="U55" s="12" t="n">
-        <v>502</v>
+        <v>553</v>
       </c>
       <c r="V55" s="13">
         <f>IFERROR(SUM(Q55:U55)/(5*P55),0)</f>
@@ -5227,25 +5227,25 @@
         <v>0</v>
       </c>
       <c r="O56" s="12" t="n">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="P56" s="12" t="n">
-        <v>1249</v>
+        <v>1456</v>
       </c>
       <c r="Q56" s="12" t="n">
-        <v>870</v>
+        <v>1008</v>
       </c>
       <c r="R56" s="12" t="n">
-        <v>1191</v>
+        <v>1388</v>
       </c>
       <c r="S56" s="12" t="n">
-        <v>1220</v>
+        <v>1421</v>
       </c>
       <c r="T56" s="12" t="n">
-        <v>1249</v>
+        <v>1456</v>
       </c>
       <c r="U56" s="12" t="n">
-        <v>820</v>
+        <v>935</v>
       </c>
       <c r="V56" s="13">
         <f>IFERROR(SUM(Q56:U56)/(5*P56),0)</f>
@@ -5314,25 +5314,25 @@
         <v>0</v>
       </c>
       <c r="O57" s="12" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="P57" s="12" t="n">
-        <v>291</v>
+        <v>430</v>
       </c>
       <c r="Q57" s="12" t="n">
-        <v>256</v>
+        <v>332</v>
       </c>
       <c r="R57" s="12" t="n">
-        <v>288</v>
+        <v>422</v>
       </c>
       <c r="S57" s="12" t="n">
-        <v>289</v>
+        <v>420</v>
       </c>
       <c r="T57" s="12" t="n">
-        <v>291</v>
+        <v>430</v>
       </c>
       <c r="U57" s="12" t="n">
-        <v>269</v>
+        <v>338</v>
       </c>
       <c r="V57" s="13">
         <f>IFERROR(SUM(Q57:U57)/(5*P57),0)</f>
@@ -5401,25 +5401,25 @@
         <v>0</v>
       </c>
       <c r="O58" s="12" t="n">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="P58" s="12" t="n">
-        <v>861</v>
+        <v>1119</v>
       </c>
       <c r="Q58" s="12" t="n">
-        <v>549</v>
+        <v>715</v>
       </c>
       <c r="R58" s="12" t="n">
-        <v>838</v>
+        <v>1087</v>
       </c>
       <c r="S58" s="12" t="n">
-        <v>847</v>
+        <v>1099</v>
       </c>
       <c r="T58" s="12" t="n">
-        <v>861</v>
+        <v>1119</v>
       </c>
       <c r="U58" s="12" t="n">
-        <v>583</v>
+        <v>760</v>
       </c>
       <c r="V58" s="13">
         <f>IFERROR(SUM(Q58:U58)/(5*P58),0)</f>
@@ -5488,25 +5488,25 @@
         <v>0</v>
       </c>
       <c r="O59" s="12" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P59" s="12" t="n">
-        <v>219</v>
+        <v>374</v>
       </c>
       <c r="Q59" s="12" t="n">
-        <v>131</v>
+        <v>188</v>
       </c>
       <c r="R59" s="12" t="n">
-        <v>212</v>
+        <v>361</v>
       </c>
       <c r="S59" s="12" t="n">
-        <v>216</v>
+        <v>362</v>
       </c>
       <c r="T59" s="12" t="n">
-        <v>219</v>
+        <v>374</v>
       </c>
       <c r="U59" s="12" t="n">
-        <v>115</v>
+        <v>177</v>
       </c>
       <c r="V59" s="13">
         <f>IFERROR(SUM(Q59:U59)/(5*P59),0)</f>
@@ -5575,25 +5575,25 @@
         <v>0</v>
       </c>
       <c r="O60" s="12" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="P60" s="12" t="n">
+        <v>393</v>
+      </c>
+      <c r="Q60" s="12" t="n">
+        <v>280</v>
+      </c>
+      <c r="R60" s="12" t="n">
+        <v>386</v>
+      </c>
+      <c r="S60" s="12" t="n">
+        <v>385</v>
+      </c>
+      <c r="T60" s="12" t="n">
+        <v>393</v>
+      </c>
+      <c r="U60" s="12" t="n">
         <v>254</v>
-      </c>
-      <c r="Q60" s="12" t="n">
-        <v>202</v>
-      </c>
-      <c r="R60" s="12" t="n">
-        <v>248</v>
-      </c>
-      <c r="S60" s="12" t="n">
-        <v>250</v>
-      </c>
-      <c r="T60" s="12" t="n">
-        <v>254</v>
-      </c>
-      <c r="U60" s="12" t="n">
-        <v>169</v>
       </c>
       <c r="V60" s="13">
         <f>IFERROR(SUM(Q60:U60)/(5*P60),0)</f>
@@ -5662,25 +5662,25 @@
         <v>0</v>
       </c>
       <c r="O61" s="12" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="P61" s="12" t="n">
-        <v>207</v>
+        <v>349</v>
       </c>
       <c r="Q61" s="12" t="n">
-        <v>181</v>
+        <v>271</v>
       </c>
       <c r="R61" s="12" t="n">
-        <v>205</v>
+        <v>345</v>
       </c>
       <c r="S61" s="12" t="n">
-        <v>204</v>
+        <v>342</v>
       </c>
       <c r="T61" s="12" t="n">
-        <v>207</v>
+        <v>349</v>
       </c>
       <c r="U61" s="12" t="n">
-        <v>132</v>
+        <v>215</v>
       </c>
       <c r="V61" s="13">
         <f>IFERROR(SUM(Q61:U61)/(5*P61),0)</f>
@@ -5749,25 +5749,25 @@
         <v>0</v>
       </c>
       <c r="O62" s="12" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="P62" s="12" t="n">
-        <v>171</v>
+        <v>294</v>
       </c>
       <c r="Q62" s="12" t="n">
-        <v>143</v>
+        <v>220</v>
       </c>
       <c r="R62" s="12" t="n">
-        <v>169</v>
+        <v>288</v>
       </c>
       <c r="S62" s="12" t="n">
-        <v>169</v>
+        <v>289</v>
       </c>
       <c r="T62" s="12" t="n">
-        <v>171</v>
+        <v>294</v>
       </c>
       <c r="U62" s="12" t="n">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="V62" s="13">
         <f>IFERROR(SUM(Q62:U62)/(5*P62),0)</f>
@@ -5836,25 +5836,25 @@
         <v>0</v>
       </c>
       <c r="O63" s="12" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="P63" s="12" t="n">
+        <v>225</v>
+      </c>
+      <c r="Q63" s="12" t="n">
         <v>108</v>
       </c>
-      <c r="Q63" s="12" t="n">
-        <v>71</v>
-      </c>
       <c r="R63" s="12" t="n">
-        <v>102</v>
+        <v>208</v>
       </c>
       <c r="S63" s="12" t="n">
-        <v>99</v>
+        <v>198</v>
       </c>
       <c r="T63" s="12" t="n">
-        <v>108</v>
+        <v>225</v>
       </c>
       <c r="U63" s="12" t="n">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="V63" s="13">
         <f>IFERROR(SUM(Q63:U63)/(5*P63),0)</f>
@@ -5923,25 +5923,25 @@
         <v>0</v>
       </c>
       <c r="O64" s="12" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="P64" s="12" t="n">
-        <v>826</v>
+        <v>943</v>
       </c>
       <c r="Q64" s="12" t="n">
-        <v>577</v>
+        <v>639</v>
       </c>
       <c r="R64" s="12" t="n">
-        <v>801</v>
+        <v>915</v>
       </c>
       <c r="S64" s="12" t="n">
-        <v>807</v>
+        <v>918</v>
       </c>
       <c r="T64" s="12" t="n">
-        <v>826</v>
+        <v>943</v>
       </c>
       <c r="U64" s="12" t="n">
-        <v>532</v>
+        <v>585</v>
       </c>
       <c r="V64" s="13">
         <f>IFERROR(SUM(Q64:U64)/(5*P64),0)</f>
@@ -6010,25 +6010,25 @@
         <v>0</v>
       </c>
       <c r="O65" s="12" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P65" s="12" t="n">
-        <v>232</v>
+        <v>374</v>
       </c>
       <c r="Q65" s="12" t="n">
-        <v>150</v>
+        <v>192</v>
       </c>
       <c r="R65" s="12" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="S65" s="12" t="n">
-        <v>225</v>
+        <v>353</v>
       </c>
       <c r="T65" s="12" t="n">
-        <v>232</v>
+        <v>374</v>
       </c>
       <c r="U65" s="12" t="n">
-        <v>219</v>
+        <v>294</v>
       </c>
       <c r="V65" s="13">
         <f>IFERROR(SUM(Q65:U65)/(5*P65),0)</f>
@@ -6097,25 +6097,25 @@
         <v>0</v>
       </c>
       <c r="O66" s="12" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="P66" s="12" t="n">
-        <v>882</v>
+        <v>1026</v>
       </c>
       <c r="Q66" s="12" t="n">
-        <v>395</v>
+        <v>419</v>
       </c>
       <c r="R66" s="12" t="n">
-        <v>859</v>
+        <v>991</v>
       </c>
       <c r="S66" s="12" t="n">
-        <v>858</v>
+        <v>985</v>
       </c>
       <c r="T66" s="12" t="n">
-        <v>882</v>
+        <v>1026</v>
       </c>
       <c r="U66" s="12" t="n">
-        <v>437</v>
+        <v>463</v>
       </c>
       <c r="V66" s="13">
         <f>IFERROR(SUM(Q66:U66)/(5*P66),0)</f>
@@ -6184,25 +6184,25 @@
         <v>0</v>
       </c>
       <c r="O67" s="12" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P67" s="12" t="n">
-        <v>234</v>
+        <v>375</v>
       </c>
       <c r="Q67" s="12" t="n">
-        <v>200</v>
+        <v>275</v>
       </c>
       <c r="R67" s="12" t="n">
-        <v>230</v>
+        <v>366</v>
       </c>
       <c r="S67" s="12" t="n">
-        <v>229</v>
+        <v>364</v>
       </c>
       <c r="T67" s="12" t="n">
-        <v>234</v>
+        <v>375</v>
       </c>
       <c r="U67" s="12" t="n">
-        <v>170</v>
+        <v>220</v>
       </c>
       <c r="V67" s="13">
         <f>IFERROR(SUM(Q67:U67)/(5*P67),0)</f>
@@ -6271,25 +6271,25 @@
         <v>0</v>
       </c>
       <c r="O68" s="12" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="P68" s="12" t="n">
-        <v>558</v>
+        <v>615</v>
       </c>
       <c r="Q68" s="12" t="n">
-        <v>362</v>
+        <v>398</v>
       </c>
       <c r="R68" s="12" t="n">
-        <v>539</v>
+        <v>593</v>
       </c>
       <c r="S68" s="12" t="n">
-        <v>535</v>
+        <v>586</v>
       </c>
       <c r="T68" s="12" t="n">
-        <v>558</v>
+        <v>615</v>
       </c>
       <c r="U68" s="12" t="n">
-        <v>365</v>
+        <v>393</v>
       </c>
       <c r="V68" s="13">
         <f>IFERROR(SUM(Q68:U68)/(5*P68),0)</f>
@@ -6358,25 +6358,25 @@
         <v>0</v>
       </c>
       <c r="O69" s="12" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="P69" s="12" t="n">
-        <v>191</v>
+        <v>316</v>
       </c>
       <c r="Q69" s="12" t="n">
-        <v>165</v>
+        <v>247</v>
       </c>
       <c r="R69" s="12" t="n">
-        <v>163</v>
+        <v>273</v>
       </c>
       <c r="S69" s="12" t="n">
-        <v>178</v>
+        <v>291</v>
       </c>
       <c r="T69" s="12" t="n">
-        <v>191</v>
+        <v>316</v>
       </c>
       <c r="U69" s="12" t="n">
-        <v>178</v>
+        <v>290</v>
       </c>
       <c r="V69" s="13">
         <f>IFERROR(SUM(Q69:U69)/(5*P69),0)</f>
@@ -6445,25 +6445,25 @@
         <v>0</v>
       </c>
       <c r="O70" s="12" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="P70" s="12" t="n">
-        <v>161</v>
+        <v>241</v>
       </c>
       <c r="Q70" s="12" t="n">
-        <v>115</v>
+        <v>151</v>
       </c>
       <c r="R70" s="12" t="n">
-        <v>153</v>
+        <v>222</v>
       </c>
       <c r="S70" s="12" t="n">
-        <v>103</v>
+        <v>144</v>
       </c>
       <c r="T70" s="12" t="n">
-        <v>161</v>
+        <v>241</v>
       </c>
       <c r="U70" s="12" t="n">
-        <v>112</v>
+        <v>168</v>
       </c>
       <c r="V70" s="13">
         <f>IFERROR(SUM(Q70:U70)/(5*P70),0)</f>
@@ -6532,25 +6532,25 @@
         <v>0</v>
       </c>
       <c r="O71" s="12" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="P71" s="12" t="n">
-        <v>201</v>
+        <v>316</v>
       </c>
       <c r="Q71" s="12" t="n">
-        <v>139</v>
+        <v>185</v>
       </c>
       <c r="R71" s="12" t="n">
-        <v>173</v>
+        <v>264</v>
       </c>
       <c r="S71" s="12" t="n">
-        <v>137</v>
+        <v>202</v>
       </c>
       <c r="T71" s="12" t="n">
-        <v>201</v>
+        <v>316</v>
       </c>
       <c r="U71" s="12" t="n">
-        <v>119</v>
+        <v>194</v>
       </c>
       <c r="V71" s="13">
         <f>IFERROR(SUM(Q71:U71)/(5*P71),0)</f>
@@ -6619,25 +6619,25 @@
         <v>0</v>
       </c>
       <c r="O72" s="12" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="P72" s="12" t="n">
-        <v>225</v>
+        <v>273</v>
       </c>
       <c r="Q72" s="12" t="n">
-        <v>194</v>
+        <v>232</v>
       </c>
       <c r="R72" s="12" t="n">
-        <v>218</v>
+        <v>264</v>
       </c>
       <c r="S72" s="12" t="n">
-        <v>220</v>
+        <v>265</v>
       </c>
       <c r="T72" s="12" t="n">
-        <v>225</v>
+        <v>273</v>
       </c>
       <c r="U72" s="12" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="V72" s="13">
         <f>IFERROR(SUM(Q72:U72)/(5*P72),0)</f>
@@ -6957,7 +6957,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>2061</v>
+        <v>1179</v>
       </c>
     </row>
   </sheetData>
@@ -6972,7 +6972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7006,7 +7006,7 @@
     <row r="2">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>chains</t>
+          <t>abu-dhabi-areas</t>
         </is>
       </c>
       <c r="B2" s="21" t="inlineStr">
@@ -7015,16 +7015,16 @@
         </is>
       </c>
       <c r="C2" s="21" t="n">
-        <v>210</v>
+        <v>324</v>
       </c>
       <c r="D2" s="21" t="n">
-        <v>2437</v>
+        <v>4132</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>full-uae</t>
+          <t>chains</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -7033,16 +7033,16 @@
         </is>
       </c>
       <c r="C3" s="21" t="n">
-        <v>1989</v>
+        <v>210</v>
       </c>
       <c r="D3" s="21" t="n">
-        <v>22182</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>more-areas</t>
+          <t>chains-2</t>
         </is>
       </c>
       <c r="B4" s="21" t="inlineStr">
@@ -7051,16 +7051,16 @@
         </is>
       </c>
       <c r="C4" s="21" t="n">
-        <v>432</v>
+        <v>330</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>6162</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>northern-emirates</t>
+          <t>full-uae</t>
         </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
@@ -7069,47 +7069,101 @@
         </is>
       </c>
       <c r="C5" s="21" t="n">
-        <v>210</v>
+        <v>1989</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>3467</v>
+        <v>22182</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
+          <t>more-areas</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>432</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>6162</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>northern-emirates</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>210</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>3467</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>northern-sparse</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>228</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>3155</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
           <t>pilot-dubai</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C9" s="21" t="n">
         <v>97</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D9" s="21" t="n">
         <v>1621</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C7" s="25">
-        <f>SUM(C2:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="25">
-        <f>SUM(D2:D6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="C10" s="25">
+        <f>SUM(C2:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="25">
+        <f>SUM(D2:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Unique places per run; the Tracker deduplicates across runs, so its total can be lower.</t>
         </is>

</xml_diff>